<commit_message>
Refactor scraper to use glob for target files and enhance data extraction; update percentile calculations and remove old targets.txt
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF248309-360A-CF4D-A896-B5CCF0DE093C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8DEE45-E057-5F48-9760-EC295F8AC8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20380" yWindow="5480" windowWidth="28040" windowHeight="17180" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Ticker</t>
   </si>
@@ -60,6 +60,18 @@
   </si>
   <si>
     <t>POSTI</t>
+  </si>
+  <si>
+    <t>MANTA</t>
+  </si>
+  <si>
+    <t>OMASP</t>
+  </si>
+  <si>
+    <t>QTCOM</t>
+  </si>
+  <si>
+    <t>AKTIA</t>
   </si>
 </sst>
 </file>
@@ -431,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -504,6 +516,62 @@
         <v>0</v>
       </c>
     </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Enhance scoring engine with risk metrics and update target files for improved stock analysis
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8DEE45-E057-5F48-9760-EC295F8AC8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2422C88E-AE94-8D44-A246-13F673E81616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20380" yWindow="5480" windowWidth="28040" windowHeight="17180" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="840" yWindow="3820" windowWidth="17560" windowHeight="17180" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Ticker</t>
   </si>
@@ -72,6 +72,45 @@
   </si>
   <si>
     <t>AKTIA</t>
+  </si>
+  <si>
+    <t>Worst Case</t>
+  </si>
+  <si>
+    <t>Probable Case</t>
+  </si>
+  <si>
+    <t>Best Case</t>
+  </si>
+  <si>
+    <t>WRT1V</t>
+  </si>
+  <si>
+    <t>KNEBV</t>
+  </si>
+  <si>
+    <t>METSO</t>
+  </si>
+  <si>
+    <t>NESTE</t>
+  </si>
+  <si>
+    <t>FORTUM</t>
+  </si>
+  <si>
+    <t>GOFORE</t>
+  </si>
+  <si>
+    <t>SAMPO</t>
+  </si>
+  <si>
+    <t>UPM</t>
+  </si>
+  <si>
+    <t>STERV</t>
+  </si>
+  <si>
+    <t>ORNBV</t>
   </si>
 </sst>
 </file>
@@ -443,10 +482,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -459,8 +498,17 @@
       <c r="D1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -473,8 +521,17 @@
       <c r="D2">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E2">
+        <v>-4.83</v>
+      </c>
+      <c r="F2">
+        <v>23.44</v>
+      </c>
+      <c r="G2">
+        <v>41.41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -487,8 +544,17 @@
       <c r="D3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E3">
+        <v>-4.1500000000000004</v>
+      </c>
+      <c r="F3">
+        <v>19.09</v>
+      </c>
+      <c r="G3">
+        <v>59.74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -501,8 +567,17 @@
       <c r="D4">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E4">
+        <v>-32.270000000000003</v>
+      </c>
+      <c r="F4">
+        <v>-2.56</v>
+      </c>
+      <c r="G4">
+        <v>28.17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -515,8 +590,17 @@
       <c r="D5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E5">
+        <v>0.49</v>
+      </c>
+      <c r="F5">
+        <v>6.86</v>
+      </c>
+      <c r="G5">
+        <v>16.12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -529,8 +613,17 @@
       <c r="D6">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E6">
+        <v>-25.51</v>
+      </c>
+      <c r="F6">
+        <v>-8.3699999999999992</v>
+      </c>
+      <c r="G6">
+        <v>7.27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -543,8 +636,17 @@
       <c r="D7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0.5</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -557,8 +659,17 @@
       <c r="D8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E8">
+        <v>-2.6</v>
+      </c>
+      <c r="F8">
+        <v>56.01</v>
+      </c>
+      <c r="G8">
+        <v>105.63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -570,6 +681,245 @@
       </c>
       <c r="D9">
         <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0.48</v>
+      </c>
+      <c r="F9">
+        <v>0.88</v>
+      </c>
+      <c r="G9">
+        <v>1.29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+      <c r="D10">
+        <v>10</v>
+      </c>
+      <c r="E10">
+        <v>-49</v>
+      </c>
+      <c r="F10">
+        <v>-2.96</v>
+      </c>
+      <c r="G10">
+        <v>27.51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <v>11</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11">
+        <v>-18.21</v>
+      </c>
+      <c r="F11">
+        <v>13.05</v>
+      </c>
+      <c r="G11">
+        <v>41.77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12">
+        <v>9</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>-13.52</v>
+      </c>
+      <c r="F12">
+        <v>18.64</v>
+      </c>
+      <c r="G12">
+        <v>48.74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>7</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>-55.07</v>
+      </c>
+      <c r="F13">
+        <v>-1.6</v>
+      </c>
+      <c r="G13">
+        <v>52.25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+      <c r="D14">
+        <v>13</v>
+      </c>
+      <c r="E14">
+        <v>-40.130000000000003</v>
+      </c>
+      <c r="F14">
+        <v>-17.82</v>
+      </c>
+      <c r="G14">
+        <v>10.15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>9.85</v>
+      </c>
+      <c r="F15">
+        <v>15.53</v>
+      </c>
+      <c r="G15">
+        <v>21.21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
+        <v>11</v>
+      </c>
+      <c r="C16">
+        <v>9</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>7.78</v>
+      </c>
+      <c r="F16">
+        <v>16.71</v>
+      </c>
+      <c r="G16">
+        <v>32.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>9</v>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <v>-18.89</v>
+      </c>
+      <c r="F17">
+        <v>3.86</v>
+      </c>
+      <c r="G17">
+        <v>23.6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18">
+        <v>11</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18">
+        <v>-18.77</v>
+      </c>
+      <c r="F18">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="G18">
+        <v>42.16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19">
+        <v>6</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>-18.28</v>
+      </c>
+      <c r="F19">
+        <v>8.4700000000000006</v>
+      </c>
+      <c r="G19">
+        <v>17.38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance scoring engine with new risk metrics and optimize scraper for improved performance
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2422C88E-AE94-8D44-A246-13F673E81616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAE024A-0454-8A47-A5B0-1A8A5A3060EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="3820" windowWidth="17560" windowHeight="17180" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="-20" yWindow="800" windowWidth="17980" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Ticker</t>
   </si>
@@ -111,6 +111,87 @@
   </si>
   <si>
     <t>ORNBV</t>
+  </si>
+  <si>
+    <t>BITTI</t>
+  </si>
+  <si>
+    <t>ELISA</t>
+  </si>
+  <si>
+    <t>TELIA1</t>
+  </si>
+  <si>
+    <t>TIETO</t>
+  </si>
+  <si>
+    <t>FSECURE</t>
+  </si>
+  <si>
+    <t>TLT1V</t>
+  </si>
+  <si>
+    <t>VINCIT</t>
+  </si>
+  <si>
+    <t>SIILI</t>
+  </si>
+  <si>
+    <t>NETUM</t>
+  </si>
+  <si>
+    <t>ALBAV</t>
+  </si>
+  <si>
+    <t>EVLI</t>
+  </si>
+  <si>
+    <t>EQV1V</t>
+  </si>
+  <si>
+    <t>ENENTO</t>
+  </si>
+  <si>
+    <t>CAPMAN</t>
+  </si>
+  <si>
+    <t>TTALO</t>
+  </si>
+  <si>
+    <t>PIHLIS</t>
+  </si>
+  <si>
+    <t>REG1V</t>
+  </si>
+  <si>
+    <t>ORIOLA</t>
+  </si>
+  <si>
+    <t>KCR</t>
+  </si>
+  <si>
+    <t>VALMT</t>
+  </si>
+  <si>
+    <t>KEMIRA</t>
+  </si>
+  <si>
+    <t>OUT1V</t>
+  </si>
+  <si>
+    <t>HUH1V</t>
+  </si>
+  <si>
+    <t>SSABBH</t>
+  </si>
+  <si>
+    <t>PAMPALO</t>
+  </si>
+  <si>
+    <t>ESENSE</t>
+  </si>
+  <si>
+    <t>MERUS</t>
   </si>
 </sst>
 </file>
@@ -482,7 +563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -636,14 +717,8 @@
       <c r="D7">
         <v>1</v>
       </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
       <c r="F7">
         <v>0.5</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -920,6 +995,576 @@
       </c>
       <c r="G19">
         <v>17.38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20">
+        <v>-5.44</v>
+      </c>
+      <c r="F20">
+        <v>3.15</v>
+      </c>
+      <c r="G20">
+        <v>14.61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21">
+        <v>7</v>
+      </c>
+      <c r="C21">
+        <v>11</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21">
+        <v>-21.8</v>
+      </c>
+      <c r="F21">
+        <v>-0.66</v>
+      </c>
+      <c r="G21">
+        <v>30.33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22">
+        <v>9</v>
+      </c>
+      <c r="C22">
+        <v>8</v>
+      </c>
+      <c r="D22">
+        <v>6</v>
+      </c>
+      <c r="E22">
+        <v>-36.5</v>
+      </c>
+      <c r="F22">
+        <v>-11.57</v>
+      </c>
+      <c r="G22">
+        <v>20.76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23">
+        <v>4</v>
+      </c>
+      <c r="C23">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23">
+        <v>-16.29</v>
+      </c>
+      <c r="F23">
+        <v>8.26</v>
+      </c>
+      <c r="G23">
+        <v>33.93</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24">
+        <v>3</v>
+      </c>
+      <c r="C24">
+        <v>3</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>6.38</v>
+      </c>
+      <c r="F24">
+        <v>20.149999999999999</v>
+      </c>
+      <c r="G24">
+        <v>31.41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>17.14</v>
+      </c>
+      <c r="F25">
+        <v>18.57</v>
+      </c>
+      <c r="G25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>11.57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="F27">
+        <v>35.979999999999997</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>-0.9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>12.61</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="F31">
+        <v>8.91</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32">
+        <v>5</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32">
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="F32">
+        <v>40.9</v>
+      </c>
+      <c r="G32">
+        <v>72.39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="F33">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34">
+        <v>4</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>20.09</v>
+      </c>
+      <c r="F34">
+        <v>27.71</v>
+      </c>
+      <c r="G34">
+        <v>38.57</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35">
+        <v>3</v>
+      </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>15.54</v>
+      </c>
+      <c r="F35">
+        <v>22.15</v>
+      </c>
+      <c r="G35">
+        <v>35.46</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36">
+        <v>7</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+      <c r="E36">
+        <v>13.66</v>
+      </c>
+      <c r="F36">
+        <v>25.9</v>
+      </c>
+      <c r="G36">
+        <v>36.61</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>20.29</v>
+      </c>
+      <c r="F37">
+        <v>22.38</v>
+      </c>
+      <c r="G37">
+        <v>25.52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38">
+        <v>5</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+      <c r="E38">
+        <v>-37.25</v>
+      </c>
+      <c r="F38">
+        <v>13.64</v>
+      </c>
+      <c r="G38">
+        <v>36.119999999999997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39">
+        <v>6</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39">
+        <v>15.56</v>
+      </c>
+      <c r="F39">
+        <v>33.1</v>
+      </c>
+      <c r="G39">
+        <v>56.83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>45</v>
+      </c>
+      <c r="B40">
+        <v>4</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="E40">
+        <v>-2.21</v>
+      </c>
+      <c r="F40">
+        <v>14.51</v>
+      </c>
+      <c r="G40">
+        <v>37.42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41">
+        <v>5</v>
+      </c>
+      <c r="C41">
+        <v>6</v>
+      </c>
+      <c r="D41">
+        <v>3</v>
+      </c>
+      <c r="E41">
+        <v>-35.090000000000003</v>
+      </c>
+      <c r="F41">
+        <v>13.8</v>
+      </c>
+      <c r="G41">
+        <v>51.45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42">
+        <v>11</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>-0.56999999999999995</v>
+      </c>
+      <c r="F42">
+        <v>29.62</v>
+      </c>
+      <c r="G42">
+        <v>43.82</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43">
+        <v>10</v>
+      </c>
+      <c r="C43">
+        <v>8</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="E43">
+        <v>-17.05</v>
+      </c>
+      <c r="F43">
+        <v>17.54</v>
+      </c>
+      <c r="G43">
+        <v>46.16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>49</v>
+      </c>
+      <c r="B44">
+        <v>2</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>20</v>
+      </c>
+      <c r="F44">
+        <v>22.86</v>
+      </c>
+      <c r="G44">
+        <v>25.71</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>50</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>44.04</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>51</v>
+      </c>
+      <c r="B46">
+        <v>2</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>11.9</v>
+      </c>
+      <c r="F46">
+        <v>15.48</v>
+      </c>
+      <c r="G46">
+        <v>19.05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance scraper with Risk vs. Reward visualization and update .gitignore to include PNG files
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAE024A-0454-8A47-A5B0-1A8A5A3060EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241F8B37-C6C3-874A-8A9A-100A1A665F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="800" windowWidth="17980" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="17980" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -594,22 +594,22 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D2">
         <v>4</v>
       </c>
       <c r="E2">
-        <v>-4.83</v>
+        <v>-19.32</v>
       </c>
       <c r="F2">
-        <v>23.44</v>
+        <v>9.01</v>
       </c>
       <c r="G2">
-        <v>41.41</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -617,22 +617,22 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>-4.1500000000000004</v>
+        <v>-16.32</v>
       </c>
       <c r="F3">
-        <v>19.09</v>
+        <v>7.11</v>
       </c>
       <c r="G3">
-        <v>59.74</v>
+        <v>39.47</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -640,22 +640,22 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4">
-        <v>-32.270000000000003</v>
+        <v>-48.14</v>
       </c>
       <c r="F4">
-        <v>-2.56</v>
+        <v>-11.46</v>
       </c>
       <c r="G4">
-        <v>28.17</v>
+        <v>30.79</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -663,7 +663,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -672,13 +672,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>0.49</v>
+        <v>3.29</v>
       </c>
       <c r="F5">
-        <v>6.86</v>
+        <v>10.68</v>
       </c>
       <c r="G5">
-        <v>16.12</v>
+        <v>17.37</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -686,22 +686,22 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>-25.51</v>
+        <v>-26.58</v>
       </c>
       <c r="F6">
-        <v>-8.3699999999999992</v>
+        <v>9.4</v>
       </c>
       <c r="G6">
-        <v>7.27</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -718,7 +718,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>0.5</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -729,19 +729,19 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
-        <v>-2.6</v>
+        <v>-21.92</v>
       </c>
       <c r="F8">
-        <v>56.01</v>
+        <v>40.549999999999997</v>
       </c>
       <c r="G8">
-        <v>105.63</v>
+        <v>97.81</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -749,22 +749,22 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>0.48</v>
+        <v>14.89</v>
       </c>
       <c r="F9">
-        <v>0.88</v>
+        <v>15.35</v>
       </c>
       <c r="G9">
-        <v>1.29</v>
+        <v>15.81</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -781,13 +781,13 @@
         <v>10</v>
       </c>
       <c r="E10">
-        <v>-49</v>
+        <v>-49.65</v>
       </c>
       <c r="F10">
-        <v>-2.96</v>
+        <v>-9.9600000000000009</v>
       </c>
       <c r="G10">
-        <v>27.51</v>
+        <v>17.48</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -795,22 +795,22 @@
         <v>16</v>
       </c>
       <c r="B11">
+        <v>11</v>
+      </c>
+      <c r="C11">
         <v>9</v>
       </c>
-      <c r="C11">
-        <v>11</v>
-      </c>
       <c r="D11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E11">
-        <v>-18.21</v>
+        <v>-16.97</v>
       </c>
       <c r="F11">
-        <v>13.05</v>
+        <v>17.07</v>
       </c>
       <c r="G11">
-        <v>41.77</v>
+        <v>54.98</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -818,22 +818,22 @@
         <v>17</v>
       </c>
       <c r="B12">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>-13.52</v>
+        <v>-11.44</v>
       </c>
       <c r="F12">
-        <v>18.64</v>
+        <v>16.62</v>
       </c>
       <c r="G12">
-        <v>48.74</v>
+        <v>46.46</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -841,22 +841,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13">
         <v>7</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13">
-        <v>-55.07</v>
+        <v>-58.8</v>
       </c>
       <c r="F13">
-        <v>-1.6</v>
+        <v>3.13</v>
       </c>
       <c r="G13">
-        <v>52.25</v>
+        <v>49.81</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -864,22 +864,22 @@
         <v>19</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D14">
         <v>13</v>
       </c>
       <c r="E14">
-        <v>-40.130000000000003</v>
+        <v>-41.7</v>
       </c>
       <c r="F14">
-        <v>-17.82</v>
+        <v>-16.18</v>
       </c>
       <c r="G14">
-        <v>10.15</v>
+        <v>7.28</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -896,13 +896,13 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>9.85</v>
+        <v>33.159999999999997</v>
       </c>
       <c r="F15">
-        <v>15.53</v>
+        <v>28.87</v>
       </c>
       <c r="G15">
-        <v>21.21</v>
+        <v>24.57</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -913,19 +913,19 @@
         <v>11</v>
       </c>
       <c r="C16">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>7.78</v>
+        <v>7.46</v>
       </c>
       <c r="F16">
-        <v>16.71</v>
+        <v>18.64</v>
       </c>
       <c r="G16">
-        <v>32.25</v>
+        <v>35.590000000000003</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -933,7 +933,7 @@
         <v>22</v>
       </c>
       <c r="B17">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17">
         <v>5</v>
@@ -942,13 +942,13 @@
         <v>4</v>
       </c>
       <c r="E17">
-        <v>-18.89</v>
+        <v>-22.65</v>
       </c>
       <c r="F17">
-        <v>3.86</v>
+        <v>6.87</v>
       </c>
       <c r="G17">
-        <v>23.6</v>
+        <v>49.2</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -956,22 +956,22 @@
         <v>23</v>
       </c>
       <c r="B18">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18">
         <v>3</v>
       </c>
       <c r="E18">
-        <v>-18.77</v>
+        <v>-15.43</v>
       </c>
       <c r="F18">
-        <v>19.010000000000002</v>
+        <v>24.52</v>
       </c>
       <c r="G18">
-        <v>42.16</v>
+        <v>47.99</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -988,13 +988,13 @@
         <v>1</v>
       </c>
       <c r="E19">
-        <v>-18.28</v>
+        <v>-19.940000000000001</v>
       </c>
       <c r="F19">
-        <v>8.4700000000000006</v>
+        <v>9.5299999999999994</v>
       </c>
       <c r="G19">
-        <v>17.38</v>
+        <v>17.899999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1002,22 +1002,22 @@
         <v>25</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20">
-        <v>-5.44</v>
+        <v>-2.21</v>
       </c>
       <c r="F20">
-        <v>3.15</v>
+        <v>10.41</v>
       </c>
       <c r="G20">
-        <v>14.61</v>
+        <v>26.18</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1025,22 +1025,22 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C21">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D21">
         <v>5</v>
       </c>
       <c r="E21">
-        <v>-21.8</v>
+        <v>-19.21</v>
       </c>
       <c r="F21">
-        <v>-0.66</v>
+        <v>2.25</v>
       </c>
       <c r="G21">
-        <v>30.33</v>
+        <v>28.21</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1048,22 +1048,22 @@
         <v>27</v>
       </c>
       <c r="B22">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C22">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D22">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E22">
-        <v>-36.5</v>
+        <v>-35.590000000000003</v>
       </c>
       <c r="F22">
-        <v>-11.57</v>
+        <v>-4.97</v>
       </c>
       <c r="G22">
-        <v>20.76</v>
+        <v>23.84</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1071,22 +1071,22 @@
         <v>28</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C23">
         <v>6</v>
       </c>
       <c r="D23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23">
-        <v>-16.29</v>
+        <v>-13.16</v>
       </c>
       <c r="F23">
-        <v>8.26</v>
+        <v>3.58</v>
       </c>
       <c r="G23">
-        <v>33.93</v>
+        <v>26.32</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1103,13 +1103,13 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>6.38</v>
+        <v>-3.63</v>
       </c>
       <c r="F24">
-        <v>20.149999999999999</v>
+        <v>8.84</v>
       </c>
       <c r="G24">
-        <v>31.41</v>
+        <v>19.05</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1126,13 +1126,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>17.14</v>
+        <v>19.53</v>
       </c>
       <c r="F25">
-        <v>18.57</v>
+        <v>20.99</v>
       </c>
       <c r="G25">
-        <v>20</v>
+        <v>22.45</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1149,7 +1149,7 @@
         <v>1</v>
       </c>
       <c r="F26">
-        <v>11.57</v>
+        <v>20.77</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1166,7 +1166,7 @@
         <v>0</v>
       </c>
       <c r="F27">
-        <v>35.979999999999997</v>
+        <v>18.47</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1183,7 +1183,7 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>-0.9</v>
+        <v>-8.6999999999999993</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1214,7 +1214,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>12.61</v>
+        <v>13.04</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1230,8 +1230,14 @@
       <c r="D31">
         <v>2</v>
       </c>
+      <c r="E31">
+        <v>1.42</v>
+      </c>
       <c r="F31">
-        <v>8.91</v>
+        <v>6.49</v>
+      </c>
+      <c r="G31">
+        <v>11.56</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1239,22 +1245,22 @@
         <v>37</v>
       </c>
       <c r="B32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32">
         <v>0</v>
       </c>
       <c r="E32">
-        <v>19.399999999999999</v>
+        <v>2.1</v>
       </c>
       <c r="F32">
-        <v>40.9</v>
+        <v>19.25</v>
       </c>
       <c r="G32">
-        <v>72.39</v>
+        <v>42.95</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1271,7 +1277,7 @@
         <v>0</v>
       </c>
       <c r="F33">
-        <v>25</v>
+        <v>22.95</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1279,22 +1285,22 @@
         <v>39</v>
       </c>
       <c r="B34">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C34">
         <v>1</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34">
-        <v>20.09</v>
+        <v>1.28</v>
       </c>
       <c r="F34">
-        <v>27.71</v>
+        <v>20.77</v>
       </c>
       <c r="G34">
-        <v>38.57</v>
+        <v>34.619999999999997</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1302,22 +1308,22 @@
         <v>40</v>
       </c>
       <c r="B35">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C35">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
       <c r="E35">
-        <v>15.54</v>
+        <v>4.91</v>
       </c>
       <c r="F35">
-        <v>22.15</v>
+        <v>17.68</v>
       </c>
       <c r="G35">
-        <v>35.46</v>
+        <v>29.46</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1325,22 +1331,22 @@
         <v>41</v>
       </c>
       <c r="B36">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D36">
         <v>0</v>
       </c>
       <c r="E36">
-        <v>13.66</v>
+        <v>7.91</v>
       </c>
       <c r="F36">
-        <v>25.9</v>
+        <v>33.24</v>
       </c>
       <c r="G36">
-        <v>36.61</v>
+        <v>69.06</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1357,13 +1363,13 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>20.29</v>
+        <v>8.4600000000000009</v>
       </c>
       <c r="F37">
-        <v>22.38</v>
+        <v>11.71</v>
       </c>
       <c r="G37">
-        <v>25.52</v>
+        <v>19.309999999999999</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1371,22 +1377,22 @@
         <v>43</v>
       </c>
       <c r="B38">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38">
         <v>0</v>
       </c>
       <c r="E38">
-        <v>-37.25</v>
+        <v>0.21</v>
       </c>
       <c r="F38">
-        <v>13.64</v>
+        <v>20.149999999999999</v>
       </c>
       <c r="G38">
-        <v>36.119999999999997</v>
+        <v>36.01</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1403,13 +1409,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>15.56</v>
+        <v>12.51</v>
       </c>
       <c r="F39">
-        <v>33.1</v>
+        <v>33.35</v>
       </c>
       <c r="G39">
-        <v>56.83</v>
+        <v>71.02</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1417,22 +1423,22 @@
         <v>45</v>
       </c>
       <c r="B40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C40">
         <v>2</v>
       </c>
       <c r="D40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40">
-        <v>-2.21</v>
+        <v>-3.68</v>
       </c>
       <c r="F40">
-        <v>14.51</v>
+        <v>15.64</v>
       </c>
       <c r="G40">
-        <v>37.42</v>
+        <v>51.27</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1449,13 +1455,13 @@
         <v>3</v>
       </c>
       <c r="E41">
-        <v>-35.090000000000003</v>
+        <v>-33.51</v>
       </c>
       <c r="F41">
-        <v>13.8</v>
+        <v>-4.46</v>
       </c>
       <c r="G41">
-        <v>51.45</v>
+        <v>22.48</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1463,7 +1469,7 @@
         <v>47</v>
       </c>
       <c r="B42">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C42">
         <v>2</v>
@@ -1472,13 +1478,13 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>-0.56999999999999995</v>
+        <v>17.39</v>
       </c>
       <c r="F42">
-        <v>29.62</v>
+        <v>30.08</v>
       </c>
       <c r="G42">
-        <v>43.82</v>
+        <v>43.07</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1495,13 +1501,13 @@
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-17.05</v>
+        <v>-28.4</v>
       </c>
       <c r="F43">
-        <v>17.54</v>
+        <v>6.48</v>
       </c>
       <c r="G43">
-        <v>46.16</v>
+        <v>27.46</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1518,13 +1524,13 @@
         <v>0</v>
       </c>
       <c r="E44">
-        <v>20</v>
+        <v>230.88</v>
       </c>
       <c r="F44">
-        <v>22.86</v>
+        <v>238.76</v>
       </c>
       <c r="G44">
-        <v>25.71</v>
+        <v>246.64</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1541,7 +1547,7 @@
         <v>0</v>
       </c>
       <c r="F45">
-        <v>44.04</v>
+        <v>56.06</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1558,13 +1564,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>11.9</v>
+        <v>8.0500000000000007</v>
       </c>
       <c r="F46">
-        <v>15.48</v>
+        <v>11.49</v>
       </c>
       <c r="G46">
-        <v>19.05</v>
+        <v>14.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Manual Analyst Ratings spreadsheet to reflect latest data
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241F8B37-C6C3-874A-8A9A-100A1A665F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CFDECCE-328F-434B-8CCB-D118F5D8EE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="17980" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -594,22 +594,22 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2">
-        <v>-19.32</v>
+        <v>-19.809999999999999</v>
       </c>
       <c r="F2">
-        <v>9.01</v>
+        <v>6.34</v>
       </c>
       <c r="G2">
-        <v>25.7</v>
+        <v>19.989999999999998</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -617,22 +617,22 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3">
         <v>3</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>-16.32</v>
+        <v>-8.19</v>
       </c>
       <c r="F3">
-        <v>7.11</v>
+        <v>14.23</v>
       </c>
       <c r="G3">
-        <v>39.47</v>
+        <v>33.89</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -640,22 +640,22 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4">
-        <v>-48.14</v>
+        <v>-58.14</v>
       </c>
       <c r="F4">
-        <v>-11.46</v>
+        <v>-9.6999999999999993</v>
       </c>
       <c r="G4">
-        <v>30.79</v>
+        <v>53.78</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -672,13 +672,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>3.29</v>
+        <v>-5.68</v>
       </c>
       <c r="F5">
-        <v>10.68</v>
+        <v>1.07</v>
       </c>
       <c r="G5">
-        <v>17.37</v>
+        <v>7.18</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -686,22 +686,22 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>-26.58</v>
+        <v>-8.26</v>
       </c>
       <c r="F6">
-        <v>9.4</v>
+        <v>7.52</v>
       </c>
       <c r="G6">
-        <v>7.2</v>
+        <v>28.44</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -718,7 +718,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>0.67</v>
+        <v>4.3499999999999996</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -726,22 +726,22 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8">
-        <v>-21.92</v>
+        <v>-33.229999999999997</v>
       </c>
       <c r="F8">
-        <v>40.549999999999997</v>
+        <v>26.58</v>
       </c>
       <c r="G8">
-        <v>97.81</v>
+        <v>64.22</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -749,22 +749,22 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C9">
         <v>0</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>14.89</v>
+        <v>0.87</v>
       </c>
       <c r="F9">
-        <v>15.35</v>
+        <v>2.61</v>
       </c>
       <c r="G9">
-        <v>15.81</v>
+        <v>4.3499999999999996</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -772,22 +772,22 @@
         <v>15</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E10">
-        <v>-49.65</v>
+        <v>-45.95</v>
       </c>
       <c r="F10">
-        <v>-9.9600000000000009</v>
+        <v>-1.77</v>
       </c>
       <c r="G10">
-        <v>17.48</v>
+        <v>26.13</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -804,13 +804,13 @@
         <v>3</v>
       </c>
       <c r="E11">
-        <v>-16.97</v>
+        <v>-7.81</v>
       </c>
       <c r="F11">
-        <v>17.07</v>
+        <v>28.52</v>
       </c>
       <c r="G11">
-        <v>54.98</v>
+        <v>72.099999999999994</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -827,13 +827,13 @@
         <v>1</v>
       </c>
       <c r="E12">
-        <v>-11.44</v>
+        <v>-15.91</v>
       </c>
       <c r="F12">
-        <v>16.62</v>
+        <v>11.06</v>
       </c>
       <c r="G12">
-        <v>46.46</v>
+        <v>39.07</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -841,22 +841,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D13">
         <v>3</v>
       </c>
       <c r="E13">
-        <v>-58.8</v>
+        <v>-55.23</v>
       </c>
       <c r="F13">
-        <v>3.13</v>
+        <v>15.32</v>
       </c>
       <c r="G13">
-        <v>49.81</v>
+        <v>96.08</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -867,19 +867,19 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D14">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14">
-        <v>-41.7</v>
+        <v>-37.090000000000003</v>
       </c>
       <c r="F14">
-        <v>-16.18</v>
+        <v>-8.76</v>
       </c>
       <c r="G14">
-        <v>7.28</v>
+        <v>15.75</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -893,16 +893,16 @@
         <v>0</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15">
-        <v>33.159999999999997</v>
+        <v>45.58</v>
       </c>
       <c r="F15">
-        <v>28.87</v>
+        <v>50.6</v>
       </c>
       <c r="G15">
-        <v>24.57</v>
+        <v>55.62</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -910,22 +910,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C16">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>7.46</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="F16">
-        <v>18.64</v>
+        <v>16.14</v>
       </c>
       <c r="G16">
-        <v>35.590000000000003</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -933,22 +933,22 @@
         <v>22</v>
       </c>
       <c r="B17">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D17">
         <v>4</v>
       </c>
       <c r="E17">
-        <v>-22.65</v>
+        <v>-18.86</v>
       </c>
       <c r="F17">
-        <v>6.87</v>
+        <v>14.76</v>
       </c>
       <c r="G17">
-        <v>49.2</v>
+        <v>58.93</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -956,22 +956,22 @@
         <v>23</v>
       </c>
       <c r="B18">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C18">
         <v>5</v>
       </c>
       <c r="D18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>-15.43</v>
+        <v>-15.25</v>
       </c>
       <c r="F18">
-        <v>24.52</v>
+        <v>22.78</v>
       </c>
       <c r="G18">
-        <v>47.99</v>
+        <v>48.31</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -988,13 +988,13 @@
         <v>1</v>
       </c>
       <c r="E19">
-        <v>-19.940000000000001</v>
+        <v>-18.149999999999999</v>
       </c>
       <c r="F19">
-        <v>9.5299999999999994</v>
+        <v>11.8</v>
       </c>
       <c r="G19">
-        <v>17.899999999999999</v>
+        <v>20.54</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1011,13 +1011,13 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>-2.21</v>
+        <v>-1.9</v>
       </c>
       <c r="F20">
-        <v>10.41</v>
+        <v>10.76</v>
       </c>
       <c r="G20">
-        <v>26.18</v>
+        <v>26.58</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1028,19 +1028,19 @@
         <v>6</v>
       </c>
       <c r="C21">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D21">
         <v>5</v>
       </c>
       <c r="E21">
-        <v>-19.21</v>
+        <v>-11.12</v>
       </c>
       <c r="F21">
-        <v>2.25</v>
+        <v>10.54</v>
       </c>
       <c r="G21">
-        <v>28.21</v>
+        <v>41.03</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1051,19 +1051,19 @@
         <v>4</v>
       </c>
       <c r="C22">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E22">
-        <v>-35.590000000000003</v>
+        <v>-37.08</v>
       </c>
       <c r="F22">
-        <v>-4.97</v>
+        <v>-6.41</v>
       </c>
       <c r="G22">
-        <v>23.84</v>
+        <v>23.14</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1071,7 +1071,7 @@
         <v>28</v>
       </c>
       <c r="B23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C23">
         <v>6</v>
@@ -1080,13 +1080,13 @@
         <v>2</v>
       </c>
       <c r="E23">
-        <v>-13.16</v>
+        <v>-12.56</v>
       </c>
       <c r="F23">
-        <v>3.58</v>
+        <v>5.25</v>
       </c>
       <c r="G23">
-        <v>26.32</v>
+        <v>27.19</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1103,13 +1103,13 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>-3.63</v>
+        <v>-15.21</v>
       </c>
       <c r="F24">
-        <v>8.84</v>
+        <v>-1.75</v>
       </c>
       <c r="G24">
-        <v>19.05</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1126,13 +1126,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>19.53</v>
+        <v>15.82</v>
       </c>
       <c r="F25">
-        <v>20.99</v>
+        <v>17.23</v>
       </c>
       <c r="G25">
-        <v>22.45</v>
+        <v>18.64</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1149,7 +1149,7 @@
         <v>1</v>
       </c>
       <c r="F26">
-        <v>20.77</v>
+        <v>35.57</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1163,10 +1163,10 @@
         <v>0</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27">
-        <v>18.47</v>
+        <v>49.12</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1183,7 +1183,7 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>-8.6999999999999993</v>
+        <v>-0.47</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1214,7 +1214,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>13.04</v>
+        <v>10.64</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1230,14 +1230,8 @@
       <c r="D31">
         <v>2</v>
       </c>
-      <c r="E31">
-        <v>1.42</v>
-      </c>
       <c r="F31">
-        <v>6.49</v>
-      </c>
-      <c r="G31">
-        <v>11.56</v>
+        <v>6.38</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1254,13 +1248,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>2.1</v>
+        <v>15.22</v>
       </c>
       <c r="F32">
-        <v>19.25</v>
+        <v>34.57</v>
       </c>
       <c r="G32">
-        <v>42.95</v>
+        <v>61.31</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1274,10 +1268,16 @@
         <v>0</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E33">
+        <v>21.11</v>
       </c>
       <c r="F33">
-        <v>22.95</v>
+        <v>23.99</v>
+      </c>
+      <c r="G33">
+        <v>26.87</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1285,22 +1285,22 @@
         <v>39</v>
       </c>
       <c r="B34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34">
-        <v>1.28</v>
+        <v>5.05</v>
       </c>
       <c r="F34">
-        <v>20.77</v>
+        <v>22.87</v>
       </c>
       <c r="G34">
-        <v>34.619999999999997</v>
+        <v>39.630000000000003</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1317,13 +1317,13 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>4.91</v>
+        <v>13.2</v>
       </c>
       <c r="F35">
-        <v>17.68</v>
+        <v>26.97</v>
       </c>
       <c r="G35">
-        <v>29.46</v>
+        <v>39.69</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1331,7 +1331,7 @@
         <v>41</v>
       </c>
       <c r="B36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -1340,13 +1340,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>7.91</v>
+        <v>20.77</v>
       </c>
       <c r="F36">
-        <v>33.24</v>
+        <v>41.06</v>
       </c>
       <c r="G36">
-        <v>69.06</v>
+        <v>61.03</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1354,7 +1354,7 @@
         <v>42</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C37">
         <v>2</v>
@@ -1362,14 +1362,8 @@
       <c r="D37">
         <v>0</v>
       </c>
-      <c r="E37">
-        <v>8.4600000000000009</v>
-      </c>
       <c r="F37">
-        <v>11.71</v>
-      </c>
-      <c r="G37">
-        <v>19.309999999999999</v>
+        <v>13.38</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1386,13 +1380,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>0.21</v>
+        <v>5.69</v>
       </c>
       <c r="F38">
-        <v>20.149999999999999</v>
+        <v>22.85</v>
       </c>
       <c r="G38">
-        <v>36.01</v>
+        <v>38.479999999999997</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1409,13 +1403,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>12.51</v>
+        <v>13.84</v>
       </c>
       <c r="F39">
-        <v>33.35</v>
+        <v>34.93</v>
       </c>
       <c r="G39">
-        <v>71.02</v>
+        <v>73.040000000000006</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1432,13 +1426,13 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-3.68</v>
+        <v>-0.47</v>
       </c>
       <c r="F40">
-        <v>15.64</v>
+        <v>15.69</v>
       </c>
       <c r="G40">
-        <v>51.27</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1449,19 +1443,19 @@
         <v>5</v>
       </c>
       <c r="C41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D41">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E41">
-        <v>-33.51</v>
+        <v>-32.26</v>
       </c>
       <c r="F41">
-        <v>-4.46</v>
+        <v>3.92</v>
       </c>
       <c r="G41">
-        <v>22.48</v>
+        <v>35.47</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1478,13 +1472,13 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>17.39</v>
+        <v>17.420000000000002</v>
       </c>
       <c r="F42">
-        <v>30.08</v>
+        <v>32.58</v>
       </c>
       <c r="G42">
-        <v>43.07</v>
+        <v>47.73</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1492,22 +1486,22 @@
         <v>48</v>
       </c>
       <c r="B43">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C43">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D43">
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-28.4</v>
+        <v>-37.15</v>
       </c>
       <c r="F43">
-        <v>6.48</v>
+        <v>-0.28000000000000003</v>
       </c>
       <c r="G43">
-        <v>27.46</v>
+        <v>43.84</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1515,22 +1509,16 @@
         <v>49</v>
       </c>
       <c r="B44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C44">
         <v>0</v>
       </c>
       <c r="D44">
-        <v>0</v>
-      </c>
-      <c r="E44">
-        <v>230.88</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>238.76</v>
-      </c>
-      <c r="G44">
-        <v>246.64</v>
+        <v>28.65</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1544,10 +1532,10 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F45">
-        <v>56.06</v>
+        <v>35.06</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1564,13 +1552,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>8.0500000000000007</v>
+        <v>-0.84</v>
       </c>
       <c r="F46">
-        <v>11.49</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="G46">
-        <v>14.94</v>
+        <v>5.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update target files: add new entries for energy, industrial, pharma, consumer, and real estate sectors; remove outdated entries
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CFDECCE-328F-434B-8CCB-D118F5D8EE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1357CD5A-F43D-2B4A-A9F5-B3DCE590C411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="17980" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Ticker</t>
   </si>
@@ -192,6 +192,48 @@
   </si>
   <si>
     <t>MERUS</t>
+  </si>
+  <si>
+    <t>SOSI1</t>
+  </si>
+  <si>
+    <t>METSB</t>
+  </si>
+  <si>
+    <t>EXEL</t>
+  </si>
+  <si>
+    <t>SCANFL</t>
+  </si>
+  <si>
+    <t>GLA1V</t>
+  </si>
+  <si>
+    <t>VIK1V</t>
+  </si>
+  <si>
+    <t>HEALTH</t>
+  </si>
+  <si>
+    <t>TOIVO</t>
+  </si>
+  <si>
+    <t>INVEST</t>
+  </si>
+  <si>
+    <t>TOKMAN</t>
+  </si>
+  <si>
+    <t>PUUILO</t>
+  </si>
+  <si>
+    <t>OLVAS</t>
+  </si>
+  <si>
+    <t>HKFOODS</t>
+  </si>
+  <si>
+    <t>KESKOA</t>
   </si>
 </sst>
 </file>
@@ -563,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -603,13 +645,13 @@
         <v>3</v>
       </c>
       <c r="E2">
-        <v>-19.809999999999999</v>
+        <v>-19.71</v>
       </c>
       <c r="F2">
-        <v>6.34</v>
+        <v>6.83</v>
       </c>
       <c r="G2">
-        <v>19.989999999999998</v>
+        <v>20.13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -626,13 +668,13 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>-8.19</v>
+        <v>-2.2799999999999998</v>
       </c>
       <c r="F3">
-        <v>14.23</v>
+        <v>20.440000000000001</v>
       </c>
       <c r="G3">
-        <v>33.89</v>
+        <v>42.51</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -649,13 +691,13 @@
         <v>7</v>
       </c>
       <c r="E4">
-        <v>-58.14</v>
+        <v>-55.58</v>
       </c>
       <c r="F4">
-        <v>-9.6999999999999993</v>
+        <v>-0.82</v>
       </c>
       <c r="G4">
-        <v>53.78</v>
+        <v>63.19</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -672,13 +714,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>-5.68</v>
+        <v>-10.57</v>
       </c>
       <c r="F5">
-        <v>1.07</v>
+        <v>-4.17</v>
       </c>
       <c r="G5">
-        <v>7.18</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -695,13 +737,13 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>-8.26</v>
+        <v>-8.84</v>
       </c>
       <c r="F6">
-        <v>7.52</v>
+        <v>6.84</v>
       </c>
       <c r="G6">
-        <v>28.44</v>
+        <v>27.62</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -718,7 +760,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>4.3499999999999996</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -735,13 +777,13 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>-33.229999999999997</v>
+        <v>-34.14</v>
       </c>
       <c r="F8">
-        <v>26.58</v>
+        <v>24.85</v>
       </c>
       <c r="G8">
-        <v>64.22</v>
+        <v>61.98</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -757,14 +799,8 @@
       <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9">
-        <v>0.87</v>
-      </c>
       <c r="F9">
-        <v>2.61</v>
-      </c>
-      <c r="G9">
-        <v>4.3499999999999996</v>
+        <v>5.26</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -772,22 +808,22 @@
         <v>15</v>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10">
-        <v>-45.95</v>
+        <v>-43.91</v>
       </c>
       <c r="F10">
-        <v>-1.77</v>
+        <v>3.9</v>
       </c>
       <c r="G10">
-        <v>26.13</v>
+        <v>30.88</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -795,22 +831,22 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D11">
         <v>3</v>
       </c>
       <c r="E11">
-        <v>-7.81</v>
+        <v>-10.71</v>
       </c>
       <c r="F11">
-        <v>28.52</v>
+        <v>25.54</v>
       </c>
       <c r="G11">
-        <v>72.099999999999994</v>
+        <v>66.67</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -827,13 +863,13 @@
         <v>1</v>
       </c>
       <c r="E12">
-        <v>-15.91</v>
+        <v>-13.96</v>
       </c>
       <c r="F12">
-        <v>11.06</v>
+        <v>14.4</v>
       </c>
       <c r="G12">
-        <v>39.07</v>
+        <v>42.29</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -841,22 +877,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D13">
         <v>3</v>
       </c>
       <c r="E13">
-        <v>-55.23</v>
+        <v>-56.3</v>
       </c>
       <c r="F13">
-        <v>15.32</v>
+        <v>12.06</v>
       </c>
       <c r="G13">
-        <v>96.08</v>
+        <v>80.569999999999993</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -870,16 +906,16 @@
         <v>10</v>
       </c>
       <c r="D14">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E14">
-        <v>-37.090000000000003</v>
+        <v>-36.9</v>
       </c>
       <c r="F14">
-        <v>-8.76</v>
+        <v>-8.3800000000000008</v>
       </c>
       <c r="G14">
-        <v>15.75</v>
+        <v>16.100000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -896,13 +932,13 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>45.58</v>
+        <v>47.96</v>
       </c>
       <c r="F15">
-        <v>50.6</v>
+        <v>53.06</v>
       </c>
       <c r="G15">
-        <v>55.62</v>
+        <v>58.16</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -910,7 +946,7 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16">
         <v>6</v>
@@ -919,13 +955,13 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>4.6900000000000004</v>
+        <v>2.57</v>
       </c>
       <c r="F16">
-        <v>16.14</v>
+        <v>13.78</v>
       </c>
       <c r="G16">
-        <v>26.6</v>
+        <v>24.03</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -936,19 +972,19 @@
         <v>11</v>
       </c>
       <c r="C17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D17">
         <v>4</v>
       </c>
       <c r="E17">
-        <v>-18.86</v>
+        <v>-15.1</v>
       </c>
       <c r="F17">
-        <v>14.76</v>
+        <v>18.420000000000002</v>
       </c>
       <c r="G17">
-        <v>58.93</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -959,19 +995,19 @@
         <v>12</v>
       </c>
       <c r="C18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18">
-        <v>-15.25</v>
+        <v>-12.99</v>
       </c>
       <c r="F18">
-        <v>22.78</v>
+        <v>26.28</v>
       </c>
       <c r="G18">
-        <v>48.31</v>
+        <v>52.27</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -988,13 +1024,13 @@
         <v>1</v>
       </c>
       <c r="E19">
-        <v>-18.149999999999999</v>
+        <v>-23.24</v>
       </c>
       <c r="F19">
-        <v>11.8</v>
+        <v>4.8600000000000003</v>
       </c>
       <c r="G19">
-        <v>20.54</v>
+        <v>13.05</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1011,13 +1047,13 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>-1.9</v>
+        <v>-2.36</v>
       </c>
       <c r="F20">
-        <v>10.76</v>
+        <v>10.24</v>
       </c>
       <c r="G20">
-        <v>26.58</v>
+        <v>25.98</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1034,13 +1070,13 @@
         <v>5</v>
       </c>
       <c r="E21">
-        <v>-11.12</v>
+        <v>-5.92</v>
       </c>
       <c r="F21">
-        <v>10.54</v>
+        <v>17.46</v>
       </c>
       <c r="G21">
-        <v>41.03</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1051,19 +1087,19 @@
         <v>4</v>
       </c>
       <c r="C22">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E22">
-        <v>-37.08</v>
+        <v>-32.950000000000003</v>
       </c>
       <c r="F22">
-        <v>-6.41</v>
+        <v>2.15</v>
       </c>
       <c r="G22">
-        <v>23.14</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1080,13 +1116,13 @@
         <v>2</v>
       </c>
       <c r="E23">
-        <v>-12.56</v>
+        <v>-8.8800000000000008</v>
       </c>
       <c r="F23">
-        <v>5.25</v>
+        <v>11.56</v>
       </c>
       <c r="G23">
-        <v>27.19</v>
+        <v>36.67</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1103,13 +1139,13 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>-15.21</v>
+        <v>-16.670000000000002</v>
       </c>
       <c r="F24">
-        <v>-1.75</v>
+        <v>1.96</v>
       </c>
       <c r="G24">
-        <v>4.74</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1126,13 +1162,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>15.82</v>
+        <v>18.16</v>
       </c>
       <c r="F25">
-        <v>17.23</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="G25">
-        <v>18.64</v>
+        <v>21.04</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1149,7 +1185,7 @@
         <v>1</v>
       </c>
       <c r="F26">
-        <v>35.57</v>
+        <v>38.58</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1166,7 +1202,7 @@
         <v>1</v>
       </c>
       <c r="F27">
-        <v>49.12</v>
+        <v>25.93</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1183,7 +1219,7 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>-0.47</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1214,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>10.64</v>
+        <v>8.7899999999999991</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1231,7 +1267,7 @@
         <v>2</v>
       </c>
       <c r="F31">
-        <v>6.38</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1248,13 +1284,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>15.22</v>
+        <v>15.06</v>
       </c>
       <c r="F32">
-        <v>34.57</v>
+        <v>34.380000000000003</v>
       </c>
       <c r="G32">
-        <v>61.31</v>
+        <v>61.09</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1271,13 +1307,13 @@
         <v>1</v>
       </c>
       <c r="E33">
-        <v>21.11</v>
+        <v>20.14</v>
       </c>
       <c r="F33">
-        <v>23.99</v>
+        <v>23</v>
       </c>
       <c r="G33">
-        <v>26.87</v>
+        <v>25.86</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1294,13 +1330,13 @@
         <v>2</v>
       </c>
       <c r="E34">
-        <v>5.05</v>
+        <v>2.86</v>
       </c>
       <c r="F34">
-        <v>22.87</v>
+        <v>20.309999999999999</v>
       </c>
       <c r="G34">
-        <v>39.630000000000003</v>
+        <v>36.72</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1308,22 +1344,22 @@
         <v>40</v>
       </c>
       <c r="B35">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
       <c r="E35">
-        <v>13.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="F35">
-        <v>26.97</v>
+        <v>24.16</v>
       </c>
       <c r="G35">
-        <v>39.69</v>
+        <v>34.76</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1340,13 +1376,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>20.77</v>
+        <v>22.35</v>
       </c>
       <c r="F36">
-        <v>41.06</v>
+        <v>42.9</v>
       </c>
       <c r="G36">
-        <v>61.03</v>
+        <v>63.13</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1354,7 +1390,7 @@
         <v>42</v>
       </c>
       <c r="B37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C37">
         <v>2</v>
@@ -1362,8 +1398,14 @@
       <c r="D37">
         <v>0</v>
       </c>
+      <c r="E37">
+        <v>2.75</v>
+      </c>
       <c r="F37">
-        <v>13.38</v>
+        <v>4.87</v>
+      </c>
+      <c r="G37">
+        <v>5.93</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1380,13 +1422,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>5.69</v>
+        <v>9.52</v>
       </c>
       <c r="F38">
-        <v>22.85</v>
+        <v>27.3</v>
       </c>
       <c r="G38">
-        <v>38.479999999999997</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1403,13 +1445,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>13.84</v>
+        <v>17.920000000000002</v>
       </c>
       <c r="F39">
-        <v>34.93</v>
+        <v>38.58</v>
       </c>
       <c r="G39">
-        <v>73.040000000000006</v>
+        <v>79.25</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1426,13 +1468,13 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-0.47</v>
+        <v>-2.62</v>
       </c>
       <c r="F40">
-        <v>15.69</v>
+        <v>18.75</v>
       </c>
       <c r="G40">
-        <v>49.3</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1446,16 +1488,16 @@
         <v>5</v>
       </c>
       <c r="D41">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E41">
-        <v>-32.26</v>
+        <v>-23.69</v>
       </c>
       <c r="F41">
-        <v>3.92</v>
+        <v>19.88</v>
       </c>
       <c r="G41">
-        <v>35.47</v>
+        <v>52.61</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1472,13 +1514,13 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>17.420000000000002</v>
+        <v>17.78</v>
       </c>
       <c r="F42">
-        <v>32.58</v>
+        <v>32.979999999999997</v>
       </c>
       <c r="G42">
-        <v>47.73</v>
+        <v>48.18</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1489,19 +1531,19 @@
         <v>12</v>
       </c>
       <c r="C43">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D43">
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-37.15</v>
+        <v>-34.200000000000003</v>
       </c>
       <c r="F43">
-        <v>-0.28000000000000003</v>
+        <v>9.3800000000000008</v>
       </c>
       <c r="G43">
-        <v>43.84</v>
+        <v>50.49</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1509,7 +1551,7 @@
         <v>49</v>
       </c>
       <c r="B44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -1518,7 +1560,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>28.65</v>
+        <v>26.44</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1535,7 +1577,7 @@
         <v>1</v>
       </c>
       <c r="F45">
-        <v>35.06</v>
+        <v>37.200000000000003</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1552,13 +1594,293 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>-0.84</v>
+        <v>-9.6199999999999992</v>
       </c>
       <c r="F46">
-        <v>2.3199999999999998</v>
+        <v>-6.73</v>
       </c>
       <c r="G46">
-        <v>5.49</v>
+        <v>-3.85</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>52</v>
+      </c>
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="F47">
+        <v>-15.38</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>53</v>
+      </c>
+      <c r="B48">
+        <v>2</v>
+      </c>
+      <c r="C48">
+        <v>4</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48">
+        <v>-6.99</v>
+      </c>
+      <c r="F48">
+        <v>10.49</v>
+      </c>
+      <c r="G48">
+        <v>19.05</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>54</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>-12.5</v>
+      </c>
+      <c r="F49">
+        <v>-10.42</v>
+      </c>
+      <c r="G49">
+        <v>-8.33</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>55</v>
+      </c>
+      <c r="B50">
+        <v>0</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <v>2</v>
+      </c>
+      <c r="F50">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>56</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>20.93</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>57</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>488.24</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>58</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53">
+        <v>0</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>54.53</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>59</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54">
+        <v>0</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>28.76</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>60</v>
+      </c>
+      <c r="B55">
+        <v>0</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>1</v>
+      </c>
+      <c r="F55">
+        <v>-1.41</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56">
+        <v>1</v>
+      </c>
+      <c r="C56">
+        <v>4</v>
+      </c>
+      <c r="D56">
+        <v>2</v>
+      </c>
+      <c r="E56">
+        <v>-9.92</v>
+      </c>
+      <c r="F56">
+        <v>-4.71</v>
+      </c>
+      <c r="G56">
+        <v>-1.48</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57">
+        <v>6</v>
+      </c>
+      <c r="C57">
+        <v>1</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57">
+        <v>-6.99</v>
+      </c>
+      <c r="F57">
+        <v>-2.71</v>
+      </c>
+      <c r="G57">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>63</v>
+      </c>
+      <c r="B58">
+        <v>2</v>
+      </c>
+      <c r="C58">
+        <v>3</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <v>-6.1</v>
+      </c>
+      <c r="F58">
+        <v>6.42</v>
+      </c>
+      <c r="G58">
+        <v>25.2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>64</v>
+      </c>
+      <c r="B59">
+        <v>1</v>
+      </c>
+      <c r="C59">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59">
+        <v>5.59</v>
+      </c>
+      <c r="F59">
+        <v>16.77</v>
+      </c>
+      <c r="G59">
+        <v>27.33</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>65</v>
+      </c>
+      <c r="B60">
+        <v>5</v>
+      </c>
+      <c r="C60">
+        <v>1</v>
+      </c>
+      <c r="D60">
+        <v>1</v>
+      </c>
+      <c r="E60">
+        <v>-2.2599999999999998</v>
+      </c>
+      <c r="F60">
+        <v>10.96</v>
+      </c>
+      <c r="G60">
+        <v>18.309999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update targets_consumer.txt to add NOHO and ensure newline at end of file
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1357CD5A-F43D-2B4A-A9F5-B3DCE590C411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E1D07D-0128-F842-9AD5-AF7CC8D6EA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17980" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
   <si>
     <t>Ticker</t>
   </si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t>KESKOA</t>
+  </si>
+  <si>
+    <t>NOHO</t>
   </si>
 </sst>
 </file>
@@ -605,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -645,13 +648,13 @@
         <v>3</v>
       </c>
       <c r="E2">
-        <v>-19.71</v>
+        <v>-21.43</v>
       </c>
       <c r="F2">
-        <v>6.83</v>
+        <v>4.78</v>
       </c>
       <c r="G2">
-        <v>20.13</v>
+        <v>17.559999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -668,13 +671,13 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>-2.2799999999999998</v>
+        <v>-2.68</v>
       </c>
       <c r="F3">
-        <v>20.440000000000001</v>
+        <v>19.95</v>
       </c>
       <c r="G3">
-        <v>42.51</v>
+        <v>41.93</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -694,7 +697,7 @@
         <v>-55.58</v>
       </c>
       <c r="F4">
-        <v>-0.82</v>
+        <v>1.27</v>
       </c>
       <c r="G4">
         <v>63.19</v>
@@ -714,13 +717,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>-10.57</v>
+        <v>-10.84</v>
       </c>
       <c r="F5">
-        <v>-4.17</v>
+        <v>-4.46</v>
       </c>
       <c r="G5">
-        <v>1.63</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -737,13 +740,13 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>-8.84</v>
+        <v>-8.42</v>
       </c>
       <c r="F6">
-        <v>6.84</v>
+        <v>7.33</v>
       </c>
       <c r="G6">
-        <v>27.62</v>
+        <v>28.21</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -760,7 +763,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>3.45</v>
+        <v>6.01</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -777,13 +780,13 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>-34.14</v>
+        <v>-34.54</v>
       </c>
       <c r="F8">
-        <v>24.85</v>
+        <v>23.73</v>
       </c>
       <c r="G8">
-        <v>61.98</v>
+        <v>60.47</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -800,7 +803,7 @@
         <v>1</v>
       </c>
       <c r="F9">
-        <v>5.26</v>
+        <v>6.38</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -817,13 +820,13 @@
         <v>8</v>
       </c>
       <c r="E10">
-        <v>-43.91</v>
+        <v>-43.56</v>
       </c>
       <c r="F10">
-        <v>3.9</v>
+        <v>4.55</v>
       </c>
       <c r="G10">
-        <v>30.88</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -840,13 +843,13 @@
         <v>3</v>
       </c>
       <c r="E11">
-        <v>-10.71</v>
+        <v>-11.07</v>
       </c>
       <c r="F11">
-        <v>25.54</v>
+        <v>24.86</v>
       </c>
       <c r="G11">
-        <v>66.67</v>
+        <v>66.010000000000005</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -857,19 +860,19 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12">
-        <v>-13.96</v>
+        <v>-17.510000000000002</v>
       </c>
       <c r="F12">
-        <v>14.4</v>
+        <v>9.58</v>
       </c>
       <c r="G12">
-        <v>42.29</v>
+        <v>36.42</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -886,13 +889,13 @@
         <v>3</v>
       </c>
       <c r="E13">
-        <v>-56.3</v>
+        <v>-56.6</v>
       </c>
       <c r="F13">
-        <v>12.06</v>
+        <v>11.48</v>
       </c>
       <c r="G13">
-        <v>80.569999999999993</v>
+        <v>79.34</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -903,19 +906,19 @@
         <v>0</v>
       </c>
       <c r="C14">
+        <v>9</v>
+      </c>
+      <c r="D14">
         <v>10</v>
       </c>
-      <c r="D14">
-        <v>11</v>
-      </c>
       <c r="E14">
-        <v>-36.9</v>
+        <v>-37.119999999999997</v>
       </c>
       <c r="F14">
-        <v>-8.3800000000000008</v>
+        <v>-9.31</v>
       </c>
       <c r="G14">
-        <v>16.100000000000001</v>
+        <v>15.69</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -932,13 +935,13 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>47.96</v>
+        <v>48.26</v>
       </c>
       <c r="F15">
-        <v>53.06</v>
+        <v>53.37</v>
       </c>
       <c r="G15">
-        <v>58.16</v>
+        <v>58.49</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -955,13 +958,13 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>2.57</v>
+        <v>2.2599999999999998</v>
       </c>
       <c r="F16">
-        <v>13.78</v>
+        <v>13.44</v>
       </c>
       <c r="G16">
-        <v>24.03</v>
+        <v>23.66</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -978,13 +981,13 @@
         <v>4</v>
       </c>
       <c r="E17">
-        <v>-15.1</v>
+        <v>-15.98</v>
       </c>
       <c r="F17">
-        <v>18.420000000000002</v>
+        <v>17.190000000000001</v>
       </c>
       <c r="G17">
-        <v>66.3</v>
+        <v>64.569999999999993</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1001,13 +1004,13 @@
         <v>1</v>
       </c>
       <c r="E18">
-        <v>-12.99</v>
+        <v>-14.07</v>
       </c>
       <c r="F18">
-        <v>26.28</v>
+        <v>24.7</v>
       </c>
       <c r="G18">
-        <v>52.27</v>
+        <v>50.38</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1024,13 +1027,13 @@
         <v>1</v>
       </c>
       <c r="E19">
-        <v>-23.24</v>
+        <v>-21.99</v>
       </c>
       <c r="F19">
-        <v>4.8600000000000003</v>
+        <v>6.57</v>
       </c>
       <c r="G19">
-        <v>13.05</v>
+        <v>14.89</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1047,13 +1050,13 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>-2.36</v>
+        <v>-7.32</v>
       </c>
       <c r="F20">
-        <v>10.24</v>
+        <v>4.63</v>
       </c>
       <c r="G20">
-        <v>25.98</v>
+        <v>19.579999999999998</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1070,13 +1073,13 @@
         <v>5</v>
       </c>
       <c r="E21">
-        <v>-5.92</v>
+        <v>-3.97</v>
       </c>
       <c r="F21">
-        <v>17.46</v>
+        <v>19.75</v>
       </c>
       <c r="G21">
-        <v>49.3</v>
+        <v>52.39</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1093,13 +1096,13 @@
         <v>7</v>
       </c>
       <c r="E22">
-        <v>-32.950000000000003</v>
+        <v>-31.44</v>
       </c>
       <c r="F22">
-        <v>2.15</v>
+        <v>4.5599999999999996</v>
       </c>
       <c r="G22">
-        <v>31.2</v>
+        <v>34.159999999999997</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1116,13 +1119,13 @@
         <v>2</v>
       </c>
       <c r="E23">
-        <v>-8.8800000000000008</v>
+        <v>-11.11</v>
       </c>
       <c r="F23">
-        <v>11.56</v>
+        <v>8.17</v>
       </c>
       <c r="G23">
-        <v>36.67</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1185,7 +1188,7 @@
         <v>1</v>
       </c>
       <c r="F26">
-        <v>38.58</v>
+        <v>36.76</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1202,7 +1205,7 @@
         <v>1</v>
       </c>
       <c r="F27">
-        <v>25.93</v>
+        <v>25.46</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1219,7 +1222,7 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>2.94</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1250,7 +1253,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>8.7899999999999991</v>
+        <v>6.56</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1267,7 +1270,7 @@
         <v>2</v>
       </c>
       <c r="F31">
-        <v>2.04</v>
+        <v>3.09</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1284,13 +1287,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>15.06</v>
+        <v>13.32</v>
       </c>
       <c r="F32">
-        <v>34.380000000000003</v>
+        <v>32.35</v>
       </c>
       <c r="G32">
-        <v>61.09</v>
+        <v>58.65</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1307,13 +1310,13 @@
         <v>1</v>
       </c>
       <c r="E33">
-        <v>20.14</v>
+        <v>19.73</v>
       </c>
       <c r="F33">
-        <v>23</v>
+        <v>22.58</v>
       </c>
       <c r="G33">
-        <v>25.86</v>
+        <v>25.43</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1330,13 +1333,13 @@
         <v>2</v>
       </c>
       <c r="E34">
-        <v>2.86</v>
+        <v>4.22</v>
       </c>
       <c r="F34">
-        <v>20.309999999999999</v>
+        <v>21.9</v>
       </c>
       <c r="G34">
-        <v>36.72</v>
+        <v>38.520000000000003</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1353,13 +1356,13 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>9.1999999999999993</v>
+        <v>13.2</v>
       </c>
       <c r="F35">
-        <v>24.16</v>
+        <v>28.71</v>
       </c>
       <c r="G35">
-        <v>34.76</v>
+        <v>39.69</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1376,13 +1379,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>22.35</v>
+        <v>20</v>
       </c>
       <c r="F36">
-        <v>42.9</v>
+        <v>40.159999999999997</v>
       </c>
       <c r="G36">
-        <v>63.13</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1399,13 +1402,13 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>2.75</v>
+        <v>0.94</v>
       </c>
       <c r="F37">
-        <v>4.87</v>
+        <v>3.02</v>
       </c>
       <c r="G37">
-        <v>5.93</v>
+        <v>4.0599999999999996</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1422,13 +1425,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>9.52</v>
+        <v>6.23</v>
       </c>
       <c r="F38">
-        <v>27.3</v>
+        <v>23.48</v>
       </c>
       <c r="G38">
-        <v>43.5</v>
+        <v>39.19</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1445,13 +1448,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>17.920000000000002</v>
+        <v>17.37</v>
       </c>
       <c r="F39">
-        <v>38.58</v>
+        <v>37.61</v>
       </c>
       <c r="G39">
-        <v>79.25</v>
+        <v>78.400000000000006</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1468,13 +1471,13 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-2.62</v>
+        <v>-1.78</v>
       </c>
       <c r="F40">
-        <v>18.75</v>
+        <v>19.77</v>
       </c>
       <c r="G40">
-        <v>55.2</v>
+        <v>56.54</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1491,13 +1494,13 @@
         <v>3</v>
       </c>
       <c r="E41">
-        <v>-23.69</v>
+        <v>-28.23</v>
       </c>
       <c r="F41">
-        <v>19.88</v>
+        <v>11.8</v>
       </c>
       <c r="G41">
-        <v>52.61</v>
+        <v>43.53</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1514,13 +1517,13 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>17.78</v>
+        <v>18.14</v>
       </c>
       <c r="F42">
-        <v>32.979999999999997</v>
+        <v>33.380000000000003</v>
       </c>
       <c r="G42">
-        <v>48.18</v>
+        <v>48.63</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1537,13 +1540,13 @@
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-34.200000000000003</v>
+        <v>-37.1</v>
       </c>
       <c r="F43">
-        <v>9.3800000000000008</v>
+        <v>4.63</v>
       </c>
       <c r="G43">
-        <v>50.49</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1560,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>26.44</v>
+        <v>25.28</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1577,7 +1580,7 @@
         <v>1</v>
       </c>
       <c r="F45">
-        <v>37.200000000000003</v>
+        <v>37.57</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1594,13 +1597,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>-9.6199999999999992</v>
+        <v>-8.1999999999999993</v>
       </c>
       <c r="F46">
-        <v>-6.73</v>
+        <v>-5.27</v>
       </c>
       <c r="G46">
-        <v>-3.85</v>
+        <v>-2.34</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1617,7 +1620,7 @@
         <v>1</v>
       </c>
       <c r="F47">
-        <v>-15.38</v>
+        <v>-14.25</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1634,13 +1637,13 @@
         <v>2</v>
       </c>
       <c r="E48">
-        <v>-6.99</v>
+        <v>-6.92</v>
       </c>
       <c r="F48">
-        <v>10.49</v>
+        <v>10.57</v>
       </c>
       <c r="G48">
-        <v>19.05</v>
+        <v>19.14</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1657,13 +1660,13 @@
         <v>0</v>
       </c>
       <c r="E49">
-        <v>-12.5</v>
+        <v>-13.58</v>
       </c>
       <c r="F49">
-        <v>-10.42</v>
+        <v>-11.52</v>
       </c>
       <c r="G49">
-        <v>-8.33</v>
+        <v>-9.4700000000000006</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1680,7 +1683,7 @@
         <v>2</v>
       </c>
       <c r="F50">
-        <v>0.16</v>
+        <v>8.51</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1697,7 +1700,7 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>20.93</v>
+        <v>17.649999999999999</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -1714,7 +1717,7 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>488.24</v>
+        <v>485.37</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -1731,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>54.53</v>
+        <v>59.82</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -1748,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>28.76</v>
+        <v>32.450000000000003</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -1765,7 +1768,7 @@
         <v>1</v>
       </c>
       <c r="F55">
-        <v>-1.41</v>
+        <v>-1.96</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -1782,13 +1785,13 @@
         <v>2</v>
       </c>
       <c r="E56">
-        <v>-9.92</v>
+        <v>-8.31</v>
       </c>
       <c r="F56">
-        <v>-4.71</v>
+        <v>-3.01</v>
       </c>
       <c r="G56">
-        <v>-1.48</v>
+        <v>0.28999999999999998</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -1828,13 +1831,13 @@
         <v>0</v>
       </c>
       <c r="E58">
-        <v>-6.1</v>
+        <v>-6.25</v>
       </c>
       <c r="F58">
-        <v>6.42</v>
+        <v>6.25</v>
       </c>
       <c r="G58">
-        <v>25.2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -1851,13 +1854,13 @@
         <v>1</v>
       </c>
       <c r="E59">
-        <v>5.59</v>
+        <v>1.67</v>
       </c>
       <c r="F59">
-        <v>16.77</v>
+        <v>12.44</v>
       </c>
       <c r="G59">
-        <v>27.33</v>
+        <v>22.61</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -1874,13 +1877,36 @@
         <v>1</v>
       </c>
       <c r="E60">
-        <v>-2.2599999999999998</v>
+        <v>-2.06</v>
       </c>
       <c r="F60">
-        <v>10.96</v>
+        <v>11.19</v>
       </c>
       <c r="G60">
-        <v>18.309999999999999</v>
+        <v>18.559999999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>66</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+      <c r="C61">
+        <v>0</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>12.88</v>
+      </c>
+      <c r="F61">
+        <v>16.47</v>
+      </c>
+      <c r="G61">
+        <v>22.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Manual analyst ratings updated.
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E1D07D-0128-F842-9AD5-AF7CC8D6EA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3601A6-39A9-4442-8F73-04DBCD4F0D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17980" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
@@ -648,13 +648,13 @@
         <v>3</v>
       </c>
       <c r="E2">
-        <v>-21.43</v>
+        <v>-21.14</v>
       </c>
       <c r="F2">
-        <v>4.78</v>
+        <v>6.73</v>
       </c>
       <c r="G2">
-        <v>17.559999999999999</v>
+        <v>19.37</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -671,13 +671,13 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>-2.68</v>
+        <v>5.82</v>
       </c>
       <c r="F3">
-        <v>19.95</v>
+        <v>30.42</v>
       </c>
       <c r="G3">
-        <v>41.93</v>
+        <v>54.32</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -685,22 +685,22 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4">
         <v>7</v>
       </c>
       <c r="D4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4">
-        <v>-55.58</v>
+        <v>-54.52</v>
       </c>
       <c r="F4">
-        <v>1.27</v>
+        <v>3.85</v>
       </c>
       <c r="G4">
-        <v>63.19</v>
+        <v>67.05</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -717,13 +717,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>-10.84</v>
+        <v>-10.93</v>
       </c>
       <c r="F5">
-        <v>-4.46</v>
+        <v>-4.55</v>
       </c>
       <c r="G5">
-        <v>1.32</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -740,10 +740,10 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>-8.42</v>
+        <v>-12.09</v>
       </c>
       <c r="F6">
-        <v>7.33</v>
+        <v>5.13</v>
       </c>
       <c r="G6">
         <v>28.21</v>
@@ -763,7 +763,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>6.01</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -771,7 +771,7 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -780,13 +780,13 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>-34.54</v>
+        <v>-35.42</v>
       </c>
       <c r="F8">
-        <v>23.73</v>
+        <v>13.04</v>
       </c>
       <c r="G8">
-        <v>60.47</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -803,7 +803,7 @@
         <v>1</v>
       </c>
       <c r="F9">
-        <v>6.38</v>
+        <v>7.53</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -814,19 +814,19 @@
         <v>5</v>
       </c>
       <c r="C10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10">
         <v>8</v>
       </c>
       <c r="E10">
-        <v>-43.56</v>
+        <v>-40.020000000000003</v>
       </c>
       <c r="F10">
-        <v>4.55</v>
+        <v>11.56</v>
       </c>
       <c r="G10">
-        <v>31.7</v>
+        <v>39.950000000000003</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -843,13 +843,13 @@
         <v>3</v>
       </c>
       <c r="E11">
-        <v>-11.07</v>
+        <v>-8.93</v>
       </c>
       <c r="F11">
-        <v>24.86</v>
+        <v>27.61</v>
       </c>
       <c r="G11">
-        <v>66.010000000000005</v>
+        <v>70.010000000000005</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -860,19 +860,19 @@
         <v>13</v>
       </c>
       <c r="C12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>-17.510000000000002</v>
+        <v>-13.85</v>
       </c>
       <c r="F12">
-        <v>9.58</v>
+        <v>14.18</v>
       </c>
       <c r="G12">
-        <v>36.42</v>
+        <v>42.48</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -880,22 +880,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D13">
         <v>3</v>
       </c>
       <c r="E13">
-        <v>-56.6</v>
+        <v>-60.08</v>
       </c>
       <c r="F13">
-        <v>11.48</v>
+        <v>3.04</v>
       </c>
       <c r="G13">
-        <v>79.34</v>
+        <v>64.959999999999994</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -906,19 +906,19 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D14">
         <v>10</v>
       </c>
       <c r="E14">
-        <v>-37.119999999999997</v>
+        <v>-36.64</v>
       </c>
       <c r="F14">
-        <v>-9.31</v>
+        <v>-8.36</v>
       </c>
       <c r="G14">
-        <v>15.69</v>
+        <v>16.57</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -935,13 +935,13 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>48.26</v>
+        <v>45.15</v>
       </c>
       <c r="F15">
-        <v>53.37</v>
+        <v>50.15</v>
       </c>
       <c r="G15">
-        <v>58.49</v>
+        <v>55.16</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -949,22 +949,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>2.2599999999999998</v>
+        <v>-1.23</v>
       </c>
       <c r="F16">
-        <v>13.44</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="G16">
-        <v>23.66</v>
+        <v>19.440000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -981,13 +981,13 @@
         <v>4</v>
       </c>
       <c r="E17">
-        <v>-15.98</v>
+        <v>-16.02</v>
       </c>
       <c r="F17">
-        <v>17.190000000000001</v>
+        <v>16.670000000000002</v>
       </c>
       <c r="G17">
-        <v>64.569999999999993</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1004,13 +1004,13 @@
         <v>1</v>
       </c>
       <c r="E18">
-        <v>-14.07</v>
+        <v>-14.64</v>
       </c>
       <c r="F18">
-        <v>24.7</v>
+        <v>23.35</v>
       </c>
       <c r="G18">
-        <v>50.38</v>
+        <v>49.38</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1027,13 +1027,13 @@
         <v>1</v>
       </c>
       <c r="E19">
-        <v>-21.99</v>
+        <v>-20.46</v>
       </c>
       <c r="F19">
-        <v>6.57</v>
+        <v>8.65</v>
       </c>
       <c r="G19">
-        <v>14.89</v>
+        <v>17.14</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1050,13 +1050,13 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>-7.32</v>
+        <v>10.71</v>
       </c>
       <c r="F20">
-        <v>4.63</v>
+        <v>25</v>
       </c>
       <c r="G20">
-        <v>19.579999999999998</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1064,22 +1064,22 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C21">
         <v>11</v>
       </c>
       <c r="D21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21">
-        <v>-3.97</v>
+        <v>-9.39</v>
       </c>
       <c r="F21">
-        <v>19.75</v>
+        <v>12.05</v>
       </c>
       <c r="G21">
-        <v>52.39</v>
+        <v>43.79</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1096,13 +1096,13 @@
         <v>7</v>
       </c>
       <c r="E22">
-        <v>-31.44</v>
+        <v>-33.729999999999997</v>
       </c>
       <c r="F22">
-        <v>4.5599999999999996</v>
+        <v>0.83</v>
       </c>
       <c r="G22">
-        <v>34.159999999999997</v>
+        <v>29.68</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1113,19 +1113,19 @@
         <v>4</v>
       </c>
       <c r="C23">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23">
         <v>2</v>
       </c>
       <c r="E23">
-        <v>-11.11</v>
+        <v>-10.46</v>
       </c>
       <c r="F23">
-        <v>8.17</v>
+        <v>8.73</v>
       </c>
       <c r="G23">
-        <v>33.33</v>
+        <v>34.4</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1136,19 +1136,19 @@
         <v>3</v>
       </c>
       <c r="C24">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D24">
         <v>0</v>
       </c>
       <c r="E24">
-        <v>-16.670000000000002</v>
+        <v>-2.2000000000000002</v>
       </c>
       <c r="F24">
-        <v>1.96</v>
+        <v>1.71</v>
       </c>
       <c r="G24">
-        <v>2.94</v>
+        <v>7.58</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1165,13 +1165,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>18.16</v>
+        <v>16.809999999999999</v>
       </c>
       <c r="F25">
-        <v>19.600000000000001</v>
+        <v>18.23</v>
       </c>
       <c r="G25">
-        <v>21.04</v>
+        <v>19.66</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1179,16 +1179,16 @@
         <v>31</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26">
-        <v>36.76</v>
+        <v>25.82</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1205,7 +1205,7 @@
         <v>1</v>
       </c>
       <c r="F27">
-        <v>25.46</v>
+        <v>24.09</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1222,7 +1222,7 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>3.96</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1253,7 +1253,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>6.56</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1270,7 +1270,7 @@
         <v>2</v>
       </c>
       <c r="F31">
-        <v>3.09</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1287,13 +1287,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>13.32</v>
+        <v>13.79</v>
       </c>
       <c r="F32">
-        <v>32.35</v>
+        <v>32.9</v>
       </c>
       <c r="G32">
-        <v>58.65</v>
+        <v>59.31</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1310,13 +1310,13 @@
         <v>1</v>
       </c>
       <c r="E33">
-        <v>19.73</v>
+        <v>19.32</v>
       </c>
       <c r="F33">
-        <v>22.58</v>
+        <v>22.16</v>
       </c>
       <c r="G33">
-        <v>25.43</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1333,13 +1333,13 @@
         <v>2</v>
       </c>
       <c r="E34">
-        <v>4.22</v>
+        <v>3</v>
       </c>
       <c r="F34">
-        <v>21.9</v>
+        <v>20.47</v>
       </c>
       <c r="G34">
-        <v>38.520000000000003</v>
+        <v>36.9</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1356,13 +1356,13 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>13.2</v>
+        <v>11.69</v>
       </c>
       <c r="F35">
-        <v>28.71</v>
+        <v>27</v>
       </c>
       <c r="G35">
-        <v>39.69</v>
+        <v>37.83</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1379,13 +1379,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>20</v>
+        <v>19.809999999999999</v>
       </c>
       <c r="F36">
-        <v>40.159999999999997</v>
+        <v>39.94</v>
       </c>
       <c r="G36">
-        <v>60</v>
+        <v>59.74</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1402,13 +1402,13 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>0.94</v>
+        <v>4.8600000000000003</v>
       </c>
       <c r="F37">
-        <v>3.02</v>
+        <v>7.03</v>
       </c>
       <c r="G37">
-        <v>4.0599999999999996</v>
+        <v>8.11</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1425,13 +1425,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>6.23</v>
+        <v>10.35</v>
       </c>
       <c r="F38">
-        <v>23.48</v>
+        <v>28.84</v>
       </c>
       <c r="G38">
-        <v>39.19</v>
+        <v>44.6</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1448,13 +1448,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>17.37</v>
+        <v>17.809999999999999</v>
       </c>
       <c r="F39">
-        <v>37.61</v>
+        <v>38.119999999999997</v>
       </c>
       <c r="G39">
-        <v>78.400000000000006</v>
+        <v>79.08</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1471,13 +1471,13 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-1.78</v>
+        <v>-3.09</v>
       </c>
       <c r="F40">
-        <v>19.77</v>
+        <v>18.170000000000002</v>
       </c>
       <c r="G40">
-        <v>56.54</v>
+        <v>54.45</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1494,13 +1494,13 @@
         <v>3</v>
       </c>
       <c r="E41">
-        <v>-28.23</v>
+        <v>-26.14</v>
       </c>
       <c r="F41">
-        <v>11.8</v>
+        <v>10.61</v>
       </c>
       <c r="G41">
-        <v>43.53</v>
+        <v>43.94</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1508,22 +1508,22 @@
         <v>47</v>
       </c>
       <c r="B42">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D42">
         <v>0</v>
       </c>
       <c r="E42">
-        <v>18.14</v>
+        <v>3.37</v>
       </c>
       <c r="F42">
-        <v>33.380000000000003</v>
+        <v>30.17</v>
       </c>
       <c r="G42">
-        <v>48.63</v>
+        <v>45.48</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1540,13 +1540,13 @@
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-37.1</v>
+        <v>-38.67</v>
       </c>
       <c r="F43">
-        <v>4.63</v>
+        <v>6.03</v>
       </c>
       <c r="G43">
-        <v>43.9</v>
+        <v>40.299999999999997</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1563,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>25.28</v>
+        <v>35.47</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1580,7 +1580,7 @@
         <v>1</v>
       </c>
       <c r="F45">
-        <v>37.57</v>
+        <v>43.25</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1597,13 +1597,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>-8.1999999999999993</v>
+        <v>0</v>
       </c>
       <c r="F46">
-        <v>-5.27</v>
+        <v>3.19</v>
       </c>
       <c r="G46">
-        <v>-2.34</v>
+        <v>6.38</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1620,7 +1620,7 @@
         <v>1</v>
       </c>
       <c r="F47">
-        <v>-14.25</v>
+        <v>-7.61</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1628,22 +1628,22 @@
         <v>53</v>
       </c>
       <c r="B48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C48">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D48">
         <v>2</v>
       </c>
       <c r="E48">
-        <v>-6.92</v>
+        <v>-6.23</v>
       </c>
       <c r="F48">
-        <v>10.57</v>
+        <v>11.4</v>
       </c>
       <c r="G48">
-        <v>19.14</v>
+        <v>20.03</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1660,13 +1660,13 @@
         <v>0</v>
       </c>
       <c r="E49">
-        <v>-13.58</v>
+        <v>-8.6999999999999993</v>
       </c>
       <c r="F49">
-        <v>-11.52</v>
+        <v>-6.52</v>
       </c>
       <c r="G49">
-        <v>-9.4700000000000006</v>
+        <v>-4.3499999999999996</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1683,7 +1683,7 @@
         <v>2</v>
       </c>
       <c r="F50">
-        <v>8.51</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1700,7 +1700,7 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>17.649999999999999</v>
+        <v>20.37</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -1717,7 +1717,7 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>485.37</v>
+        <v>491.13</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -1734,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>59.82</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -1751,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>32.450000000000003</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -1768,7 +1768,7 @@
         <v>1</v>
       </c>
       <c r="F55">
-        <v>-1.96</v>
+        <v>-1.69</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -1785,13 +1785,13 @@
         <v>2</v>
       </c>
       <c r="E56">
-        <v>-8.31</v>
+        <v>-8.69</v>
       </c>
       <c r="F56">
-        <v>-3.01</v>
+        <v>-3.7</v>
       </c>
       <c r="G56">
-        <v>0.28999999999999998</v>
+        <v>-0.43</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -1808,13 +1808,13 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>-6.99</v>
+        <v>-3.62</v>
       </c>
       <c r="F57">
-        <v>-2.71</v>
+        <v>0.82</v>
       </c>
       <c r="G57">
-        <v>1.47</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
@@ -1831,13 +1831,13 @@
         <v>0</v>
       </c>
       <c r="E58">
-        <v>-6.25</v>
+        <v>-6.98</v>
       </c>
       <c r="F58">
-        <v>6.25</v>
+        <v>5.43</v>
       </c>
       <c r="G58">
-        <v>25</v>
+        <v>24.03</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -1854,13 +1854,13 @@
         <v>1</v>
       </c>
       <c r="E59">
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="F59">
-        <v>12.44</v>
+        <v>12.57</v>
       </c>
       <c r="G59">
-        <v>22.61</v>
+        <v>22.75</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -1877,13 +1877,13 @@
         <v>1</v>
       </c>
       <c r="E60">
-        <v>-2.06</v>
+        <v>-2.56</v>
       </c>
       <c r="F60">
-        <v>11.19</v>
+        <v>10.62</v>
       </c>
       <c r="G60">
-        <v>18.559999999999999</v>
+        <v>17.95</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
@@ -1900,13 +1900,13 @@
         <v>0</v>
       </c>
       <c r="E61">
-        <v>12.88</v>
+        <v>11.99</v>
       </c>
       <c r="F61">
-        <v>16.47</v>
+        <v>15.55</v>
       </c>
       <c r="G61">
-        <v>22.18</v>
+        <v>21.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update target files with corrected stock identifiers and URLs
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3601A6-39A9-4442-8F73-04DBCD4F0D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5C446E-6DE7-D941-A882-F8C81438B16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17980" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>Ticker</t>
   </si>
@@ -237,6 +237,36 @@
   </si>
   <si>
     <t>NOHO</t>
+  </si>
+  <si>
+    <t>KAMUX</t>
+  </si>
+  <si>
+    <t>HARVIA</t>
+  </si>
+  <si>
+    <t>MUSTI</t>
+  </si>
+  <si>
+    <t>TAALA</t>
+  </si>
+  <si>
+    <t>YIT</t>
+  </si>
+  <si>
+    <t>DIGIA</t>
+  </si>
+  <si>
+    <t>REMEDY</t>
+  </si>
+  <si>
+    <t>PON1V</t>
+  </si>
+  <si>
+    <t>CTY1S</t>
+  </si>
+  <si>
+    <t>ICP1V</t>
   </si>
 </sst>
 </file>
@@ -608,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -1909,6 +1939,200 @@
         <v>21.21</v>
       </c>
     </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>67</v>
+      </c>
+      <c r="B62">
+        <v>0</v>
+      </c>
+      <c r="C62">
+        <v>0</v>
+      </c>
+      <c r="D62">
+        <v>3</v>
+      </c>
+      <c r="E62">
+        <v>-15.25</v>
+      </c>
+      <c r="F62">
+        <v>-2.2200000000000002</v>
+      </c>
+      <c r="G62">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>68</v>
+      </c>
+      <c r="B63">
+        <v>6</v>
+      </c>
+      <c r="C63">
+        <v>1</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="F63">
+        <v>12.38</v>
+      </c>
+      <c r="G63">
+        <v>25.76</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>69</v>
+      </c>
+      <c r="B64">
+        <v>0</v>
+      </c>
+      <c r="C64">
+        <v>0</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>70</v>
+      </c>
+      <c r="B65">
+        <v>1</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>17.239999999999998</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>74</v>
+      </c>
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66">
+        <v>1</v>
+      </c>
+      <c r="D66">
+        <v>1</v>
+      </c>
+      <c r="E66">
+        <v>4.91</v>
+      </c>
+      <c r="F66">
+        <v>21.29</v>
+      </c>
+      <c r="G66">
+        <v>51.79</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>71</v>
+      </c>
+      <c r="B67">
+        <v>3</v>
+      </c>
+      <c r="C67">
+        <v>3</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67">
+        <v>1.89</v>
+      </c>
+      <c r="F67">
+        <v>7.17</v>
+      </c>
+      <c r="G67">
+        <v>20.75</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>75</v>
+      </c>
+      <c r="B68">
+        <v>0</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>72</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69">
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>27.99</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>73</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70">
+        <v>0</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70">
+        <v>27.18</v>
+      </c>
+      <c r="F70">
+        <v>30.52</v>
+      </c>
+      <c r="G70">
+        <v>33.869999999999997</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>76</v>
+      </c>
+      <c r="B71">
+        <v>1</v>
+      </c>
+      <c r="C71">
+        <v>0</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>39.369999999999997</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update SAMPO URL in targets_finance.txt for accuracy
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5C446E-6DE7-D941-A882-F8C81438B16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13C5DBD-3229-DE4C-9525-C5A0C8B32D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17980" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
@@ -982,19 +982,19 @@
         <v>15</v>
       </c>
       <c r="C16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-1.23</v>
+        <v>-1.39</v>
       </c>
       <c r="F16">
-        <v>10.199999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="G16">
-        <v>19.440000000000001</v>
+        <v>19.25</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update Manual Analyst Ratings spreadsheet
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13C5DBD-3229-DE4C-9525-C5A0C8B32D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABFA369-8A7E-A441-971A-C18B6BAEE94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17980" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
@@ -669,22 +669,22 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>-21.14</v>
+        <v>-22.34</v>
       </c>
       <c r="F2">
-        <v>6.73</v>
+        <v>5.19</v>
       </c>
       <c r="G2">
-        <v>19.37</v>
+        <v>16.489999999999998</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -692,22 +692,22 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>5.82</v>
+        <v>-2.52</v>
       </c>
       <c r="F3">
-        <v>30.42</v>
+        <v>18.93</v>
       </c>
       <c r="G3">
-        <v>54.32</v>
+        <v>42.16</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -715,22 +715,22 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
         <v>7</v>
       </c>
-      <c r="D4">
-        <v>6</v>
-      </c>
       <c r="E4">
-        <v>-54.52</v>
+        <v>-40.98</v>
       </c>
       <c r="F4">
-        <v>3.85</v>
+        <v>24.12</v>
       </c>
       <c r="G4">
-        <v>67.05</v>
+        <v>91.77</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -747,13 +747,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>-10.93</v>
+        <v>-11.91</v>
       </c>
       <c r="F5">
-        <v>-4.55</v>
+        <v>-5.61</v>
       </c>
       <c r="G5">
-        <v>1.21</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -770,13 +770,13 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>-12.09</v>
+        <v>-14.13</v>
       </c>
       <c r="F6">
-        <v>5.13</v>
+        <v>2.5</v>
       </c>
       <c r="G6">
-        <v>28.21</v>
+        <v>25.22</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -793,7 +793,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>1.07</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -810,13 +810,13 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>-35.42</v>
+        <v>-36.11</v>
       </c>
       <c r="F8">
-        <v>13.04</v>
+        <v>11.83</v>
       </c>
       <c r="G8">
-        <v>37.5</v>
+        <v>36.03</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -833,7 +833,7 @@
         <v>1</v>
       </c>
       <c r="F9">
-        <v>7.53</v>
+        <v>7.14</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -850,13 +850,13 @@
         <v>8</v>
       </c>
       <c r="E10">
-        <v>-40.020000000000003</v>
+        <v>-39.979999999999997</v>
       </c>
       <c r="F10">
-        <v>11.56</v>
+        <v>11.64</v>
       </c>
       <c r="G10">
-        <v>39.950000000000003</v>
+        <v>40.049999999999997</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -873,13 +873,13 @@
         <v>3</v>
       </c>
       <c r="E11">
-        <v>-8.93</v>
+        <v>-6.64</v>
       </c>
       <c r="F11">
-        <v>27.61</v>
+        <v>29.38</v>
       </c>
       <c r="G11">
-        <v>70.010000000000005</v>
+        <v>74.27</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -896,13 +896,13 @@
         <v>1</v>
       </c>
       <c r="E12">
-        <v>-13.85</v>
+        <v>-11.3</v>
       </c>
       <c r="F12">
-        <v>14.18</v>
+        <v>13.34</v>
       </c>
       <c r="G12">
-        <v>42.48</v>
+        <v>41.26</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -910,7 +910,7 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13">
         <v>9</v>
@@ -919,13 +919,13 @@
         <v>3</v>
       </c>
       <c r="E13">
-        <v>-60.08</v>
+        <v>-63.41</v>
       </c>
       <c r="F13">
-        <v>3.04</v>
+        <v>-2.57</v>
       </c>
       <c r="G13">
-        <v>64.959999999999994</v>
+        <v>72.36</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -942,13 +942,13 @@
         <v>10</v>
       </c>
       <c r="E14">
-        <v>-36.64</v>
+        <v>-38.21</v>
       </c>
       <c r="F14">
-        <v>-8.36</v>
+        <v>-10.78</v>
       </c>
       <c r="G14">
-        <v>16.57</v>
+        <v>13.69</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -956,7 +956,7 @@
         <v>20</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -965,13 +965,13 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>45.15</v>
+        <v>45.88</v>
       </c>
       <c r="F15">
-        <v>50.15</v>
+        <v>49.2</v>
       </c>
       <c r="G15">
-        <v>55.16</v>
+        <v>55.94</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -988,13 +988,13 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-1.39</v>
+        <v>-0.73</v>
       </c>
       <c r="F16">
-        <v>9.5</v>
+        <v>10.23</v>
       </c>
       <c r="G16">
-        <v>19.25</v>
+        <v>20.04</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1011,13 +1011,13 @@
         <v>4</v>
       </c>
       <c r="E17">
-        <v>-16.02</v>
+        <v>-18.190000000000001</v>
       </c>
       <c r="F17">
-        <v>16.670000000000002</v>
+        <v>14.78</v>
       </c>
       <c r="G17">
-        <v>64.5</v>
+        <v>61.91</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1028,19 +1028,19 @@
         <v>12</v>
       </c>
       <c r="C18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="E18">
-        <v>-14.64</v>
+        <v>-17.73</v>
       </c>
       <c r="F18">
-        <v>23.35</v>
+        <v>18.57</v>
       </c>
       <c r="G18">
-        <v>49.38</v>
+        <v>43.97</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1048,22 +1048,22 @@
         <v>24</v>
       </c>
       <c r="B19">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19">
-        <v>-20.46</v>
+        <v>-28.15</v>
       </c>
       <c r="F19">
-        <v>8.65</v>
+        <v>1.08</v>
       </c>
       <c r="G19">
-        <v>17.14</v>
+        <v>12.34</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1080,13 +1080,13 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>10.71</v>
+        <v>15.89</v>
       </c>
       <c r="F20">
-        <v>25</v>
+        <v>30.84</v>
       </c>
       <c r="G20">
-        <v>42.86</v>
+        <v>49.53</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1097,19 +1097,19 @@
         <v>7</v>
       </c>
       <c r="C21">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D21">
         <v>4</v>
       </c>
       <c r="E21">
-        <v>-9.39</v>
+        <v>-2.17</v>
       </c>
       <c r="F21">
-        <v>12.05</v>
+        <v>15.29</v>
       </c>
       <c r="G21">
-        <v>43.79</v>
+        <v>46.46</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1117,22 +1117,22 @@
         <v>27</v>
       </c>
       <c r="B22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D22">
         <v>7</v>
       </c>
       <c r="E22">
-        <v>-33.729999999999997</v>
+        <v>-31.59</v>
       </c>
       <c r="F22">
-        <v>0.83</v>
+        <v>3.84</v>
       </c>
       <c r="G22">
-        <v>29.68</v>
+        <v>33.86</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1143,19 +1143,19 @@
         <v>4</v>
       </c>
       <c r="C23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23">
         <v>2</v>
       </c>
       <c r="E23">
-        <v>-10.46</v>
+        <v>-9.5</v>
       </c>
       <c r="F23">
-        <v>8.73</v>
+        <v>9.11</v>
       </c>
       <c r="G23">
-        <v>34.4</v>
+        <v>35.75</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1163,22 +1163,22 @@
         <v>29</v>
       </c>
       <c r="B24">
+        <v>4</v>
+      </c>
+      <c r="C24">
         <v>3</v>
       </c>
-      <c r="C24">
-        <v>2</v>
-      </c>
       <c r="D24">
         <v>0</v>
       </c>
       <c r="E24">
-        <v>-2.2000000000000002</v>
+        <v>5.26</v>
       </c>
       <c r="F24">
-        <v>1.71</v>
+        <v>10</v>
       </c>
       <c r="G24">
-        <v>7.58</v>
+        <v>21.05</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1195,13 +1195,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>16.809999999999999</v>
+        <v>16.149999999999999</v>
       </c>
       <c r="F25">
-        <v>18.23</v>
+        <v>17.559999999999999</v>
       </c>
       <c r="G25">
-        <v>19.66</v>
+        <v>18.98</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1218,7 +1218,7 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>25.82</v>
+        <v>19.329999999999998</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1235,7 +1235,7 @@
         <v>1</v>
       </c>
       <c r="F27">
-        <v>24.09</v>
+        <v>13.33</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1274,7 +1274,7 @@
         <v>35</v>
       </c>
       <c r="B30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -1283,7 +1283,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>4.42</v>
+        <v>11.57</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1300,7 +1300,7 @@
         <v>2</v>
       </c>
       <c r="F31">
-        <v>2.04</v>
+        <v>4.17</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1308,7 +1308,7 @@
         <v>37</v>
       </c>
       <c r="B32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -1317,13 +1317,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>13.79</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="F32">
-        <v>32.9</v>
+        <v>22.92</v>
       </c>
       <c r="G32">
-        <v>59.31</v>
+        <v>38.340000000000003</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1340,13 +1340,13 @@
         <v>1</v>
       </c>
       <c r="E33">
-        <v>19.32</v>
+        <v>20.41</v>
       </c>
       <c r="F33">
-        <v>22.16</v>
+        <v>23.28</v>
       </c>
       <c r="G33">
-        <v>25</v>
+        <v>26.15</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1363,13 +1363,13 @@
         <v>2</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>9.35</v>
       </c>
       <c r="F34">
-        <v>20.47</v>
+        <v>29.5</v>
       </c>
       <c r="G34">
-        <v>36.9</v>
+        <v>43.88</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1386,13 +1386,13 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>11.69</v>
+        <v>11.65</v>
       </c>
       <c r="F35">
-        <v>27</v>
+        <v>26.99</v>
       </c>
       <c r="G35">
-        <v>37.83</v>
+        <v>40.78</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1409,13 +1409,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>19.809999999999999</v>
+        <v>20.58</v>
       </c>
       <c r="F36">
-        <v>39.94</v>
+        <v>40.840000000000003</v>
       </c>
       <c r="G36">
-        <v>59.74</v>
+        <v>60.77</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1432,13 +1432,13 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>4.8600000000000003</v>
+        <v>5.43</v>
       </c>
       <c r="F37">
-        <v>7.03</v>
+        <v>7.61</v>
       </c>
       <c r="G37">
-        <v>8.11</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1455,13 +1455,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>10.35</v>
+        <v>5.69</v>
       </c>
       <c r="F38">
-        <v>28.84</v>
+        <v>23.4</v>
       </c>
       <c r="G38">
-        <v>44.6</v>
+        <v>38.479999999999997</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1478,13 +1478,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>17.809999999999999</v>
+        <v>13.02</v>
       </c>
       <c r="F39">
-        <v>38.119999999999997</v>
+        <v>32.5</v>
       </c>
       <c r="G39">
-        <v>79.08</v>
+        <v>71.790000000000006</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1501,13 +1501,13 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-3.09</v>
+        <v>-4.4800000000000004</v>
       </c>
       <c r="F40">
-        <v>18.170000000000002</v>
+        <v>15.82</v>
       </c>
       <c r="G40">
-        <v>54.45</v>
+        <v>52.24</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1515,22 +1515,22 @@
         <v>46</v>
       </c>
       <c r="B41">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C41">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D41">
         <v>3</v>
       </c>
       <c r="E41">
-        <v>-26.14</v>
+        <v>-28.51</v>
       </c>
       <c r="F41">
-        <v>10.61</v>
+        <v>6.51</v>
       </c>
       <c r="G41">
-        <v>43.94</v>
+        <v>39.32</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1547,13 +1547,13 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>3.37</v>
+        <v>0.45</v>
       </c>
       <c r="F42">
-        <v>30.17</v>
+        <v>26.19</v>
       </c>
       <c r="G42">
-        <v>45.48</v>
+        <v>41.37</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1570,13 +1570,13 @@
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-38.67</v>
+        <v>-34.58</v>
       </c>
       <c r="F43">
-        <v>6.03</v>
+        <v>6.44</v>
       </c>
       <c r="G43">
-        <v>40.299999999999997</v>
+        <v>38.08</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1593,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>35.47</v>
+        <v>36.82</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1610,7 +1610,7 @@
         <v>1</v>
       </c>
       <c r="F45">
-        <v>43.25</v>
+        <v>45.66</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1627,13 +1627,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>-1.05</v>
       </c>
       <c r="F46">
-        <v>3.19</v>
+        <v>2.11</v>
       </c>
       <c r="G46">
-        <v>6.38</v>
+        <v>5.26</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1650,7 +1650,7 @@
         <v>1</v>
       </c>
       <c r="F47">
-        <v>-7.61</v>
+        <v>-9.34</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1667,13 +1667,13 @@
         <v>2</v>
       </c>
       <c r="E48">
-        <v>-6.23</v>
+        <v>-8.49</v>
       </c>
       <c r="F48">
-        <v>11.4</v>
+        <v>8.7100000000000009</v>
       </c>
       <c r="G48">
-        <v>20.03</v>
+        <v>17.13</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1690,13 +1690,13 @@
         <v>0</v>
       </c>
       <c r="E49">
-        <v>-8.6999999999999993</v>
+        <v>-9.09</v>
       </c>
       <c r="F49">
-        <v>-6.52</v>
+        <v>-6.93</v>
       </c>
       <c r="G49">
-        <v>-4.3499999999999996</v>
+        <v>-4.76</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1704,16 +1704,16 @@
         <v>55</v>
       </c>
       <c r="B50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C50">
         <v>0</v>
       </c>
       <c r="D50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50">
-        <v>6.47</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1730,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>20.37</v>
+        <v>15.56</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -1747,7 +1747,7 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>491.13</v>
+        <v>485.37</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -1764,7 +1764,7 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>65.48</v>
+        <v>69.900000000000006</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -1781,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>33.33</v>
+        <v>29.03</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -1798,7 +1798,7 @@
         <v>1</v>
       </c>
       <c r="F55">
-        <v>-1.69</v>
+        <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -1806,22 +1806,22 @@
         <v>61</v>
       </c>
       <c r="B56">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C56">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D56">
         <v>2</v>
       </c>
       <c r="E56">
-        <v>-8.69</v>
+        <v>-9.73</v>
       </c>
       <c r="F56">
-        <v>-3.7</v>
+        <v>-1.97</v>
       </c>
       <c r="G56">
-        <v>-0.43</v>
+        <v>7.19</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -1838,13 +1838,13 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>-3.62</v>
+        <v>-2.37</v>
       </c>
       <c r="F57">
-        <v>0.82</v>
+        <v>2.13</v>
       </c>
       <c r="G57">
-        <v>5.14</v>
+        <v>6.51</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
@@ -1861,13 +1861,13 @@
         <v>0</v>
       </c>
       <c r="E58">
-        <v>-6.98</v>
+        <v>0.15</v>
       </c>
       <c r="F58">
-        <v>5.43</v>
+        <v>5.46</v>
       </c>
       <c r="G58">
-        <v>24.03</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -1884,13 +1884,13 @@
         <v>1</v>
       </c>
       <c r="E59">
-        <v>1.8</v>
+        <v>-2.86</v>
       </c>
       <c r="F59">
-        <v>12.57</v>
+        <v>7.43</v>
       </c>
       <c r="G59">
-        <v>22.75</v>
+        <v>17.14</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -1907,13 +1907,13 @@
         <v>1</v>
       </c>
       <c r="E60">
-        <v>-2.56</v>
+        <v>-4.2300000000000004</v>
       </c>
       <c r="F60">
-        <v>10.62</v>
+        <v>8.3699999999999992</v>
       </c>
       <c r="G60">
-        <v>17.95</v>
+        <v>15.93</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="E61">
-        <v>11.99</v>
+        <v>15.65</v>
       </c>
       <c r="F61">
-        <v>15.55</v>
+        <v>19.32</v>
       </c>
       <c r="G61">
-        <v>21.21</v>
+        <v>25.17</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
@@ -1953,13 +1953,13 @@
         <v>3</v>
       </c>
       <c r="E62">
-        <v>-15.25</v>
+        <v>-13.91</v>
       </c>
       <c r="F62">
-        <v>-2.2200000000000002</v>
+        <v>-0.66</v>
       </c>
       <c r="G62">
-        <v>4.3</v>
+        <v>5.96</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
@@ -1976,13 +1976,13 @@
         <v>0</v>
       </c>
       <c r="E63">
-        <v>2.2999999999999998</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="F63">
-        <v>12.38</v>
+        <v>12.11</v>
       </c>
       <c r="G63">
-        <v>25.76</v>
+        <v>25.45</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
@@ -2013,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="F65">
-        <v>17.239999999999998</v>
+        <v>16.440000000000001</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
@@ -2021,22 +2021,16 @@
         <v>74</v>
       </c>
       <c r="B66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C66">
         <v>1</v>
       </c>
       <c r="D66">
-        <v>1</v>
-      </c>
-      <c r="E66">
-        <v>4.91</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>21.29</v>
-      </c>
-      <c r="G66">
-        <v>51.79</v>
+        <v>5.38</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
@@ -2053,13 +2047,13 @@
         <v>0</v>
       </c>
       <c r="E67">
-        <v>1.89</v>
+        <v>2.86</v>
       </c>
       <c r="F67">
-        <v>7.17</v>
+        <v>8.19</v>
       </c>
       <c r="G67">
-        <v>20.75</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
@@ -2090,7 +2084,7 @@
         <v>0</v>
       </c>
       <c r="F69">
-        <v>27.99</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -2130,7 +2124,7 @@
         <v>0</v>
       </c>
       <c r="F71">
-        <v>39.369999999999997</v>
+        <v>38.409999999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Manual Analyst Ratings and add new targets to industrial list
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABFA369-8A7E-A441-971A-C18B6BAEE94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AADE0928-B876-8E4F-B136-341A648F26DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17980" yWindow="780" windowWidth="18020" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="18020" yWindow="800" windowWidth="18000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t>Ticker</t>
   </si>
@@ -267,6 +267,9 @@
   </si>
   <si>
     <t>ICP1V</t>
+  </si>
+  <si>
+    <t>HIAB</t>
   </si>
 </sst>
 </file>
@@ -638,7 +641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -2127,6 +2130,29 @@
         <v>38.409999999999997</v>
       </c>
     </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>77</v>
+      </c>
+      <c r="B72">
+        <v>7</v>
+      </c>
+      <c r="C72">
+        <v>1</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72">
+        <v>-3.72</v>
+      </c>
+      <c r="F72">
+        <v>12.33</v>
+      </c>
+      <c r="G72">
+        <v>18.239999999999998</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Increase timeout for page loading and dynamic waits in scraper to enhance data retrieval reliability
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A162A06-35BC-2347-95A0-BFF1D37DD679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6467F8D-C98D-7244-8E79-61A9C6FC21F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18020" yWindow="800" windowWidth="18000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
   <si>
     <t>Ticker</t>
   </si>
@@ -273,6 +273,129 @@
   </si>
   <si>
     <t>TYRES</t>
+  </si>
+  <si>
+    <t>FSKRS</t>
+  </si>
+  <si>
+    <t>MEKKO</t>
+  </si>
+  <si>
+    <t>LINDEX</t>
+  </si>
+  <si>
+    <t>VERK</t>
+  </si>
+  <si>
+    <t>RAP1V</t>
+  </si>
+  <si>
+    <t>RAIVV</t>
+  </si>
+  <si>
+    <t>ANORA</t>
+  </si>
+  <si>
+    <t>ATRAV</t>
+  </si>
+  <si>
+    <t>APETIT</t>
+  </si>
+  <si>
+    <t>RELAIS</t>
+  </si>
+  <si>
+    <t>SANOMA</t>
+  </si>
+  <si>
+    <t>FIA1S</t>
+  </si>
+  <si>
+    <t>LAMOR</t>
+  </si>
+  <si>
+    <t>UNITED</t>
+  </si>
+  <si>
+    <t>PNA1V</t>
+  </si>
+  <si>
+    <t>KALMAR</t>
+  </si>
+  <si>
+    <t>ALMA</t>
+  </si>
+  <si>
+    <t>SUY1V</t>
+  </si>
+  <si>
+    <t>KREATE</t>
+  </si>
+  <si>
+    <t>SRV1V</t>
+  </si>
+  <si>
+    <t>ROBIT</t>
+  </si>
+  <si>
+    <t>NLG1V</t>
+  </si>
+  <si>
+    <t>BOREO</t>
+  </si>
+  <si>
+    <t>EEZY</t>
+  </si>
+  <si>
+    <t>KOSKI</t>
+  </si>
+  <si>
+    <t>FARON</t>
+  </si>
+  <si>
+    <t>NXTMH</t>
+  </si>
+  <si>
+    <t>BRETEC</t>
+  </si>
+  <si>
+    <t>BIOBV</t>
+  </si>
+  <si>
+    <t>NANOFH</t>
+  </si>
+  <si>
+    <t>LUMO</t>
+  </si>
+  <si>
+    <t>OVARO</t>
+  </si>
+  <si>
+    <t>ADMCM</t>
+  </si>
+  <si>
+    <t>SOLTEQ</t>
+  </si>
+  <si>
+    <t>SSH1V</t>
+  </si>
+  <si>
+    <t>DETEC</t>
+  </si>
+  <si>
+    <t>LEMON</t>
+  </si>
+  <si>
+    <t>LEADD</t>
+  </si>
+  <si>
+    <t>TEM1V</t>
+  </si>
+  <si>
+    <t>LOIHDE</t>
+  </si>
+  <si>
+    <t>AIFORIA</t>
   </si>
 </sst>
 </file>
@@ -644,7 +767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -684,13 +807,13 @@
         <v>4</v>
       </c>
       <c r="E2">
-        <v>-22.34</v>
+        <v>-23.17</v>
       </c>
       <c r="F2">
-        <v>5.19</v>
+        <v>4.07</v>
       </c>
       <c r="G2">
-        <v>16.489999999999998</v>
+        <v>15.25</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -698,22 +821,22 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>-2.52</v>
+        <v>-9.09</v>
       </c>
       <c r="F3">
-        <v>18.93</v>
+        <v>26.97</v>
       </c>
       <c r="G3">
-        <v>42.16</v>
+        <v>76.77</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -721,22 +844,22 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4">
-        <v>-40.98</v>
+        <v>-33.450000000000003</v>
       </c>
       <c r="F4">
-        <v>24.12</v>
+        <v>36.71</v>
       </c>
       <c r="G4">
-        <v>91.77</v>
+        <v>116.24</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -753,13 +876,13 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>-11.91</v>
+        <v>-13.39</v>
       </c>
       <c r="F5">
-        <v>-5.61</v>
+        <v>-7.19</v>
       </c>
       <c r="G5">
-        <v>0.1</v>
+        <v>-1.57</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -776,13 +899,13 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>-14.13</v>
+        <v>-14.06</v>
       </c>
       <c r="F6">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="G6">
-        <v>25.22</v>
+        <v>25.34</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -799,7 +922,7 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>0.95</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -816,13 +939,13 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <v>-36.11</v>
+        <v>-36.369999999999997</v>
       </c>
       <c r="F8">
-        <v>11.83</v>
+        <v>11.37</v>
       </c>
       <c r="G8">
-        <v>36.03</v>
+        <v>35.47</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -839,7 +962,7 @@
         <v>1</v>
       </c>
       <c r="F9">
-        <v>7.14</v>
+        <v>5.82</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -847,22 +970,22 @@
         <v>15</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C10">
         <v>8</v>
       </c>
       <c r="D10">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E10">
-        <v>-39.979999999999997</v>
+        <v>-38.130000000000003</v>
       </c>
       <c r="F10">
-        <v>11.64</v>
+        <v>8.86</v>
       </c>
       <c r="G10">
-        <v>40.049999999999997</v>
+        <v>40.020000000000003</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -870,22 +993,22 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11">
-        <v>-6.64</v>
+        <v>-9.42</v>
       </c>
       <c r="F11">
-        <v>29.38</v>
+        <v>24.13</v>
       </c>
       <c r="G11">
-        <v>74.27</v>
+        <v>67.069999999999993</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -893,22 +1016,22 @@
         <v>17</v>
       </c>
       <c r="B12">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12">
-        <v>-11.3</v>
+        <v>-18.03</v>
       </c>
       <c r="F12">
-        <v>13.34</v>
+        <v>6.98</v>
       </c>
       <c r="G12">
-        <v>41.26</v>
+        <v>30.54</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -916,22 +1039,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C13">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D13">
         <v>3</v>
       </c>
       <c r="E13">
-        <v>-63.41</v>
+        <v>-39.89</v>
       </c>
       <c r="F13">
-        <v>-2.57</v>
+        <v>7.71</v>
       </c>
       <c r="G13">
-        <v>72.36</v>
+        <v>86.21</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -948,13 +1071,13 @@
         <v>10</v>
       </c>
       <c r="E14">
-        <v>-38.21</v>
+        <v>-26.49</v>
       </c>
       <c r="F14">
-        <v>-10.78</v>
+        <v>-9.9700000000000006</v>
       </c>
       <c r="G14">
-        <v>13.69</v>
+        <v>8.5299999999999994</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -971,13 +1094,13 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>45.88</v>
+        <v>42.44</v>
       </c>
       <c r="F15">
-        <v>49.2</v>
+        <v>45.68</v>
       </c>
       <c r="G15">
-        <v>55.94</v>
+        <v>52.26</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -994,13 +1117,13 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-0.73</v>
+        <v>-1.1200000000000001</v>
       </c>
       <c r="F16">
-        <v>10.23</v>
+        <v>9.7899999999999991</v>
       </c>
       <c r="G16">
-        <v>20.04</v>
+        <v>19.57</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1017,13 +1140,13 @@
         <v>4</v>
       </c>
       <c r="E17">
-        <v>-18.190000000000001</v>
+        <v>-24.74</v>
       </c>
       <c r="F17">
-        <v>14.78</v>
+        <v>13.49</v>
       </c>
       <c r="G17">
-        <v>61.91</v>
+        <v>64.36</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1040,13 +1163,13 @@
         <v>1</v>
       </c>
       <c r="E18">
-        <v>-17.73</v>
+        <v>-17.239999999999998</v>
       </c>
       <c r="F18">
-        <v>18.57</v>
+        <v>15.46</v>
       </c>
       <c r="G18">
-        <v>43.97</v>
+        <v>39.659999999999997</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1054,7 +1177,7 @@
         <v>24</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19">
         <v>2</v>
@@ -1063,13 +1186,13 @@
         <v>2</v>
       </c>
       <c r="E19">
-        <v>-28.15</v>
+        <v>-30.47</v>
       </c>
       <c r="F19">
-        <v>1.08</v>
+        <v>-2.29</v>
       </c>
       <c r="G19">
-        <v>12.34</v>
+        <v>8.7200000000000006</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1086,13 +1209,13 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>15.89</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="F20">
-        <v>30.84</v>
+        <v>22.16</v>
       </c>
       <c r="G20">
-        <v>49.53</v>
+        <v>39.619999999999997</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1100,7 +1223,7 @@
         <v>26</v>
       </c>
       <c r="B21">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C21">
         <v>10</v>
@@ -1109,13 +1232,13 @@
         <v>4</v>
       </c>
       <c r="E21">
-        <v>-2.17</v>
+        <v>-2.85</v>
       </c>
       <c r="F21">
-        <v>15.29</v>
+        <v>15.94</v>
       </c>
       <c r="G21">
-        <v>46.46</v>
+        <v>45.43</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1132,13 +1255,13 @@
         <v>7</v>
       </c>
       <c r="E22">
-        <v>-31.59</v>
+        <v>-31.26</v>
       </c>
       <c r="F22">
-        <v>3.84</v>
+        <v>3.86</v>
       </c>
       <c r="G22">
-        <v>33.86</v>
+        <v>34.270000000000003</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1146,22 +1269,22 @@
         <v>28</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C23">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23">
-        <v>-9.5</v>
+        <v>-12.32</v>
       </c>
       <c r="F23">
-        <v>9.11</v>
+        <v>5.94</v>
       </c>
       <c r="G23">
-        <v>35.75</v>
+        <v>30.41</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1178,13 +1301,13 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>5.26</v>
+        <v>6.84</v>
       </c>
       <c r="F24">
-        <v>10</v>
+        <v>11.65</v>
       </c>
       <c r="G24">
-        <v>21.05</v>
+        <v>22.86</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1201,13 +1324,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>16.149999999999999</v>
+        <v>20.23</v>
       </c>
       <c r="F25">
-        <v>17.559999999999999</v>
+        <v>21.7</v>
       </c>
       <c r="G25">
-        <v>18.98</v>
+        <v>23.17</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1224,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>19.329999999999998</v>
+        <v>6.61</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1241,7 +1364,7 @@
         <v>1</v>
       </c>
       <c r="F27">
-        <v>13.33</v>
+        <v>12.96</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -1258,7 +1381,7 @@
         <v>1</v>
       </c>
       <c r="F28">
-        <v>5</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
@@ -1289,7 +1412,7 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>11.57</v>
+        <v>8.43</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -1323,13 +1446,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>8.6999999999999993</v>
+        <v>7.7</v>
       </c>
       <c r="F32">
-        <v>22.92</v>
+        <v>21.8</v>
       </c>
       <c r="G32">
-        <v>38.340000000000003</v>
+        <v>37.08</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1346,13 +1469,13 @@
         <v>1</v>
       </c>
       <c r="E33">
-        <v>20.41</v>
+        <v>19.59</v>
       </c>
       <c r="F33">
-        <v>23.28</v>
+        <v>22.44</v>
       </c>
       <c r="G33">
-        <v>26.15</v>
+        <v>25.28</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1369,13 +1492,13 @@
         <v>2</v>
       </c>
       <c r="E34">
-        <v>9.35</v>
+        <v>6.59</v>
       </c>
       <c r="F34">
-        <v>29.5</v>
+        <v>23.14</v>
       </c>
       <c r="G34">
-        <v>43.88</v>
+        <v>40.25</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1383,7 +1506,7 @@
         <v>40</v>
       </c>
       <c r="B35">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -1392,13 +1515,13 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>11.65</v>
+        <v>0.38</v>
       </c>
       <c r="F35">
-        <v>26.99</v>
+        <v>18.16</v>
       </c>
       <c r="G35">
-        <v>40.78</v>
+        <v>33.840000000000003</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1415,13 +1538,13 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>20.58</v>
+        <v>22.75</v>
       </c>
       <c r="F36">
-        <v>40.840000000000003</v>
+        <v>43.37</v>
       </c>
       <c r="G36">
-        <v>60.77</v>
+        <v>63.67</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1438,13 +1561,13 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>5.43</v>
+        <v>7.54</v>
       </c>
       <c r="F37">
-        <v>7.61</v>
+        <v>9.76</v>
       </c>
       <c r="G37">
-        <v>8.6999999999999993</v>
+        <v>10.86</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1461,13 +1584,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>5.69</v>
+        <v>8.94</v>
       </c>
       <c r="F38">
-        <v>23.4</v>
+        <v>26.63</v>
       </c>
       <c r="G38">
-        <v>38.479999999999997</v>
+        <v>42.75</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1484,13 +1607,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>13.02</v>
+        <v>-6.86</v>
       </c>
       <c r="F39">
-        <v>32.5</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="G39">
-        <v>71.790000000000006</v>
+        <v>41.58</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1498,22 +1621,22 @@
         <v>45</v>
       </c>
       <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40">
         <v>3</v>
-      </c>
-      <c r="C40">
-        <v>2</v>
       </c>
       <c r="D40">
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-4.4800000000000004</v>
+        <v>-3.56</v>
       </c>
       <c r="F40">
-        <v>15.82</v>
+        <v>11.27</v>
       </c>
       <c r="G40">
-        <v>52.24</v>
+        <v>32.61</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1530,13 +1653,13 @@
         <v>3</v>
       </c>
       <c r="E41">
-        <v>-28.51</v>
+        <v>-33.159999999999997</v>
       </c>
       <c r="F41">
-        <v>6.51</v>
+        <v>-0.77</v>
       </c>
       <c r="G41">
-        <v>39.32</v>
+        <v>30.25</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1544,22 +1667,22 @@
         <v>47</v>
       </c>
       <c r="B42">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D42">
         <v>0</v>
       </c>
       <c r="E42">
-        <v>0.45</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="F42">
-        <v>26.19</v>
+        <v>15.93</v>
       </c>
       <c r="G42">
-        <v>41.37</v>
+        <v>35.49</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1567,22 +1690,22 @@
         <v>48</v>
       </c>
       <c r="B43">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D43">
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-34.58</v>
+        <v>-35.770000000000003</v>
       </c>
       <c r="F43">
-        <v>6.44</v>
+        <v>6.28</v>
       </c>
       <c r="G43">
-        <v>38.08</v>
+        <v>35.57</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1599,7 +1722,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>36.82</v>
+        <v>41.94</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1616,7 +1739,7 @@
         <v>1</v>
       </c>
       <c r="F45">
-        <v>45.66</v>
+        <v>47.73</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1633,13 +1756,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>-1.05</v>
+        <v>1.08</v>
       </c>
       <c r="F46">
-        <v>2.11</v>
+        <v>4.3</v>
       </c>
       <c r="G46">
-        <v>5.26</v>
+        <v>7.53</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1656,7 +1779,7 @@
         <v>1</v>
       </c>
       <c r="F47">
-        <v>-9.34</v>
+        <v>-8.33</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1673,13 +1796,13 @@
         <v>2</v>
       </c>
       <c r="E48">
-        <v>-8.49</v>
+        <v>-12.83</v>
       </c>
       <c r="F48">
-        <v>8.7100000000000009</v>
+        <v>3.56</v>
       </c>
       <c r="G48">
-        <v>17.13</v>
+        <v>11.58</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1696,13 +1819,13 @@
         <v>0</v>
       </c>
       <c r="E49">
-        <v>-9.09</v>
+        <v>-6.25</v>
       </c>
       <c r="F49">
-        <v>-6.93</v>
+        <v>-4.0199999999999996</v>
       </c>
       <c r="G49">
-        <v>-4.76</v>
+        <v>-1.79</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1719,7 +1842,7 @@
         <v>1</v>
       </c>
       <c r="F50">
-        <v>2.29</v>
+        <v>6.84</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1736,7 +1859,7 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>15.56</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -1753,7 +1876,7 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>485.37</v>
+        <v>491.13</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -1770,7 +1893,7 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>69.900000000000006</v>
+        <v>64.709999999999994</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -1787,7 +1910,7 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>29.03</v>
+        <v>27.66</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -1804,7 +1927,7 @@
         <v>1</v>
       </c>
       <c r="F55">
-        <v>0.56999999999999995</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -1821,13 +1944,13 @@
         <v>2</v>
       </c>
       <c r="E56">
-        <v>-9.73</v>
+        <v>-13.34</v>
       </c>
       <c r="F56">
-        <v>-1.97</v>
+        <v>-5.89</v>
       </c>
       <c r="G56">
-        <v>7.19</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -1844,13 +1967,13 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>-2.37</v>
+        <v>-3.06</v>
       </c>
       <c r="F57">
-        <v>2.13</v>
+        <v>1.41</v>
       </c>
       <c r="G57">
-        <v>6.51</v>
+        <v>5.76</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
@@ -1858,22 +1981,16 @@
         <v>63</v>
       </c>
       <c r="B58">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D58">
         <v>0</v>
       </c>
-      <c r="E58">
-        <v>0.15</v>
-      </c>
       <c r="F58">
-        <v>5.46</v>
-      </c>
-      <c r="G58">
-        <v>21.4</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -1890,13 +2007,13 @@
         <v>1</v>
       </c>
       <c r="E59">
-        <v>-2.86</v>
+        <v>-6.08</v>
       </c>
       <c r="F59">
-        <v>7.43</v>
+        <v>3.87</v>
       </c>
       <c r="G59">
-        <v>17.14</v>
+        <v>13.26</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -1913,13 +2030,13 @@
         <v>1</v>
       </c>
       <c r="E60">
-        <v>-4.2300000000000004</v>
+        <v>-5.8</v>
       </c>
       <c r="F60">
-        <v>8.3699999999999992</v>
+        <v>5.94</v>
       </c>
       <c r="G60">
-        <v>15.93</v>
+        <v>15.94</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
@@ -1936,13 +2053,13 @@
         <v>0</v>
       </c>
       <c r="E61">
-        <v>15.65</v>
+        <v>14.56</v>
       </c>
       <c r="F61">
-        <v>19.32</v>
+        <v>18.190000000000001</v>
       </c>
       <c r="G61">
-        <v>25.17</v>
+        <v>23.99</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
@@ -1959,13 +2076,13 @@
         <v>3</v>
       </c>
       <c r="E62">
-        <v>-13.91</v>
+        <v>-14.81</v>
       </c>
       <c r="F62">
-        <v>-0.66</v>
+        <v>-1.7</v>
       </c>
       <c r="G62">
-        <v>5.96</v>
+        <v>4.8499999999999996</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
@@ -1982,13 +2099,13 @@
         <v>0</v>
       </c>
       <c r="E63">
-        <v>2.0499999999999998</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="F63">
-        <v>12.11</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="G63">
-        <v>25.45</v>
+        <v>16.96</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
@@ -2019,7 +2136,7 @@
         <v>0</v>
       </c>
       <c r="F65">
-        <v>16.440000000000001</v>
+        <v>15.65</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
@@ -2036,7 +2153,7 @@
         <v>0</v>
       </c>
       <c r="F66">
-        <v>5.38</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
@@ -2053,13 +2170,13 @@
         <v>0</v>
       </c>
       <c r="E67">
-        <v>2.86</v>
+        <v>-9.5500000000000007</v>
       </c>
       <c r="F67">
-        <v>8.19</v>
+        <v>-4.8600000000000003</v>
       </c>
       <c r="G67">
-        <v>21.9</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
@@ -2090,7 +2207,7 @@
         <v>0</v>
       </c>
       <c r="F69">
-        <v>27.55</v>
+        <v>27.99</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -2107,13 +2224,13 @@
         <v>0</v>
       </c>
       <c r="E70">
-        <v>27.18</v>
+        <v>26.67</v>
       </c>
       <c r="F70">
-        <v>30.52</v>
+        <v>30</v>
       </c>
       <c r="G70">
-        <v>33.869999999999997</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
@@ -2130,7 +2247,7 @@
         <v>0</v>
       </c>
       <c r="F71">
-        <v>38.409999999999997</v>
+        <v>63.04</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
@@ -2147,13 +2264,13 @@
         <v>0</v>
       </c>
       <c r="E72">
-        <v>-3.72</v>
+        <v>-1.83</v>
       </c>
       <c r="F72">
-        <v>12.33</v>
+        <v>13.98</v>
       </c>
       <c r="G72">
-        <v>18.239999999999998</v>
+        <v>24.79</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
@@ -2170,13 +2287,821 @@
         <v>5</v>
       </c>
       <c r="E73">
-        <v>-49.67</v>
+        <v>-49.11</v>
       </c>
       <c r="F73">
-        <v>-15.16</v>
+        <v>-14.21</v>
       </c>
       <c r="G73">
+        <v>18.97</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>79</v>
+      </c>
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74">
+        <v>2</v>
+      </c>
+      <c r="D74">
+        <v>3</v>
+      </c>
+      <c r="E74">
+        <v>-12.88</v>
+      </c>
+      <c r="F74">
+        <v>-6.06</v>
+      </c>
+      <c r="G74">
+        <v>6.06</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>80</v>
+      </c>
+      <c r="B75">
+        <v>2</v>
+      </c>
+      <c r="C75">
+        <v>1</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75">
+        <v>9.94</v>
+      </c>
+      <c r="F75">
+        <v>19.5</v>
+      </c>
+      <c r="G75">
+        <v>29.06</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>81</v>
+      </c>
+      <c r="B76">
+        <v>0</v>
+      </c>
+      <c r="C76">
+        <v>0</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>82</v>
+      </c>
+      <c r="B77">
+        <v>3</v>
+      </c>
+      <c r="C77">
+        <v>0</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
+      </c>
+      <c r="F77">
+        <v>10.34</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>83</v>
+      </c>
+      <c r="B78">
+        <v>1</v>
+      </c>
+      <c r="C78">
+        <v>0</v>
+      </c>
+      <c r="D78">
+        <v>1</v>
+      </c>
+      <c r="E78">
+        <v>-1.57</v>
+      </c>
+      <c r="F78">
+        <v>4.72</v>
+      </c>
+      <c r="G78">
+        <v>10.24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>84</v>
+      </c>
+      <c r="B79">
+        <v>5</v>
+      </c>
+      <c r="C79">
+        <v>0</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79">
+        <v>12.62</v>
+      </c>
+      <c r="F79">
+        <v>21.94</v>
+      </c>
+      <c r="G79">
+        <v>43.69</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>85</v>
+      </c>
+      <c r="B80">
+        <v>2</v>
+      </c>
+      <c r="C80">
+        <v>1</v>
+      </c>
+      <c r="D80">
+        <v>2</v>
+      </c>
+      <c r="E80">
+        <v>-9.7100000000000009</v>
+      </c>
+      <c r="F80">
+        <v>1.78</v>
+      </c>
+      <c r="G80">
         <v>17.649999999999999</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>86</v>
+      </c>
+      <c r="B81">
+        <v>3</v>
+      </c>
+      <c r="C81">
+        <v>0</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81">
+        <v>-5.33</v>
+      </c>
+      <c r="F81">
+        <v>4.91</v>
+      </c>
+      <c r="G81">
+        <v>12.43</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>87</v>
+      </c>
+      <c r="B82">
+        <v>0</v>
+      </c>
+      <c r="C82">
+        <v>0</v>
+      </c>
+      <c r="D82">
+        <v>2</v>
+      </c>
+      <c r="F82">
+        <v>2.04</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>88</v>
+      </c>
+      <c r="B83">
+        <v>2</v>
+      </c>
+      <c r="C83">
+        <v>0</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>24.57</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>89</v>
+      </c>
+      <c r="B84">
+        <v>6</v>
+      </c>
+      <c r="C84">
+        <v>1</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84">
+        <v>9.36</v>
+      </c>
+      <c r="F84">
+        <v>32.92</v>
+      </c>
+      <c r="G84">
+        <v>57.84</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>90</v>
+      </c>
+      <c r="B85">
+        <v>0</v>
+      </c>
+      <c r="C85">
+        <v>1</v>
+      </c>
+      <c r="D85">
+        <v>5</v>
+      </c>
+      <c r="E85">
+        <v>-26.05</v>
+      </c>
+      <c r="F85">
+        <v>-18.86</v>
+      </c>
+      <c r="G85">
+        <v>-3.45</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>91</v>
+      </c>
+      <c r="B86">
+        <v>0</v>
+      </c>
+      <c r="C86">
+        <v>0</v>
+      </c>
+      <c r="D86">
+        <v>2</v>
+      </c>
+      <c r="F86">
+        <v>-3.02</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>92</v>
+      </c>
+      <c r="B87">
+        <v>0</v>
+      </c>
+      <c r="C87">
+        <v>0</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>93</v>
+      </c>
+      <c r="B88">
+        <v>0</v>
+      </c>
+      <c r="C88">
+        <v>0</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="F88">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>94</v>
+      </c>
+      <c r="B89">
+        <v>5</v>
+      </c>
+      <c r="C89">
+        <v>4</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89">
+        <v>9.3800000000000008</v>
+      </c>
+      <c r="F89">
+        <v>19.22</v>
+      </c>
+      <c r="G89">
+        <v>43.23</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>95</v>
+      </c>
+      <c r="B90">
+        <v>4</v>
+      </c>
+      <c r="C90">
+        <v>1</v>
+      </c>
+      <c r="D90">
+        <v>0</v>
+      </c>
+      <c r="E90">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="F90">
+        <v>8.93</v>
+      </c>
+      <c r="G90">
+        <v>13.65</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>96</v>
+      </c>
+      <c r="B91">
+        <v>0</v>
+      </c>
+      <c r="C91">
+        <v>0</v>
+      </c>
+      <c r="D91">
+        <v>1</v>
+      </c>
+      <c r="F91">
+        <v>-13.29</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>97</v>
+      </c>
+      <c r="B92">
+        <v>3</v>
+      </c>
+      <c r="C92">
+        <v>0</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92">
+        <v>-10.71</v>
+      </c>
+      <c r="F92">
+        <v>1.18</v>
+      </c>
+      <c r="G92">
+        <v>7.14</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>98</v>
+      </c>
+      <c r="B93">
+        <v>0</v>
+      </c>
+      <c r="C93">
+        <v>0</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+      <c r="F93">
+        <v>-1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>99</v>
+      </c>
+      <c r="B94">
+        <v>2</v>
+      </c>
+      <c r="C94">
+        <v>0</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="F94">
+        <v>27.05</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>100</v>
+      </c>
+      <c r="B95">
+        <v>2</v>
+      </c>
+      <c r="C95">
+        <v>0</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="F95">
+        <v>10.32</v>
+      </c>
+      <c r="G95">
+        <v>14.61</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>101</v>
+      </c>
+      <c r="B96">
+        <v>1</v>
+      </c>
+      <c r="C96">
+        <v>0</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="F96">
+        <v>-4.28</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>102</v>
+      </c>
+      <c r="B97">
+        <v>0</v>
+      </c>
+      <c r="C97">
+        <v>0</v>
+      </c>
+      <c r="D97">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>103</v>
+      </c>
+      <c r="B98">
+        <v>1</v>
+      </c>
+      <c r="C98">
+        <v>1</v>
+      </c>
+      <c r="D98">
+        <v>1</v>
+      </c>
+      <c r="E98">
+        <v>1.43</v>
+      </c>
+      <c r="F98">
+        <v>5.61</v>
+      </c>
+      <c r="G98">
+        <v>9.7899999999999991</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>104</v>
+      </c>
+      <c r="B99">
+        <v>2</v>
+      </c>
+      <c r="C99">
+        <v>0</v>
+      </c>
+      <c r="D99">
+        <v>0</v>
+      </c>
+      <c r="E99">
+        <v>108.12</v>
+      </c>
+      <c r="F99">
+        <v>955.15</v>
+      </c>
+      <c r="G99">
+        <v>2337.04</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>105</v>
+      </c>
+      <c r="B100">
+        <v>1</v>
+      </c>
+      <c r="C100">
+        <v>0</v>
+      </c>
+      <c r="D100">
+        <v>0</v>
+      </c>
+      <c r="F100">
+        <v>11.68</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>106</v>
+      </c>
+      <c r="B101">
+        <v>1</v>
+      </c>
+      <c r="C101">
+        <v>0</v>
+      </c>
+      <c r="D101">
+        <v>0</v>
+      </c>
+      <c r="F101">
+        <v>41.51</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>107</v>
+      </c>
+      <c r="B102">
+        <v>2</v>
+      </c>
+      <c r="C102">
+        <v>0</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="F102">
+        <v>28.21</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>108</v>
+      </c>
+      <c r="B103">
+        <v>3</v>
+      </c>
+      <c r="C103">
+        <v>0</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103">
+        <v>129.88999999999999</v>
+      </c>
+      <c r="F103">
+        <v>149.43</v>
+      </c>
+      <c r="G103">
+        <v>158.62</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>109</v>
+      </c>
+      <c r="B104">
+        <v>7</v>
+      </c>
+      <c r="C104">
+        <v>3</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104">
+        <v>11.77</v>
+      </c>
+      <c r="F104">
+        <v>32.409999999999997</v>
+      </c>
+      <c r="G104">
+        <v>57.79</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>110</v>
+      </c>
+      <c r="B105">
+        <v>0</v>
+      </c>
+      <c r="C105">
+        <v>0</v>
+      </c>
+      <c r="D105">
+        <v>1</v>
+      </c>
+      <c r="F105">
+        <v>17.86</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>111</v>
+      </c>
+      <c r="B106">
+        <v>4</v>
+      </c>
+      <c r="C106">
+        <v>1</v>
+      </c>
+      <c r="D106">
+        <v>0</v>
+      </c>
+      <c r="E106">
+        <v>40.35</v>
+      </c>
+      <c r="F106">
+        <v>62.73</v>
+      </c>
+      <c r="G106">
+        <v>113.26</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>112</v>
+      </c>
+      <c r="B107">
+        <v>0</v>
+      </c>
+      <c r="C107">
+        <v>0</v>
+      </c>
+      <c r="D107">
+        <v>1</v>
+      </c>
+      <c r="F107">
+        <v>-12.5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>113</v>
+      </c>
+      <c r="B108">
+        <v>0</v>
+      </c>
+      <c r="C108">
+        <v>0</v>
+      </c>
+      <c r="D108">
+        <v>2</v>
+      </c>
+      <c r="E108">
+        <v>2.7</v>
+      </c>
+      <c r="F108">
+        <v>18.920000000000002</v>
+      </c>
+      <c r="G108">
+        <v>51.35</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>114</v>
+      </c>
+      <c r="B109">
+        <v>1</v>
+      </c>
+      <c r="C109">
+        <v>4</v>
+      </c>
+      <c r="D109">
+        <v>0</v>
+      </c>
+      <c r="E109">
+        <v>19.05</v>
+      </c>
+      <c r="F109">
+        <v>23.81</v>
+      </c>
+      <c r="G109">
+        <v>30.33</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>115</v>
+      </c>
+      <c r="B110">
+        <v>2</v>
+      </c>
+      <c r="C110">
+        <v>1</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110">
+        <v>17.77</v>
+      </c>
+      <c r="F110">
+        <v>24.84</v>
+      </c>
+      <c r="G110">
+        <v>28.48</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>116</v>
+      </c>
+      <c r="B111">
+        <v>0</v>
+      </c>
+      <c r="C111">
+        <v>0</v>
+      </c>
+      <c r="D111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>117</v>
+      </c>
+      <c r="B112">
+        <v>0</v>
+      </c>
+      <c r="C112">
+        <v>0</v>
+      </c>
+      <c r="D112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>118</v>
+      </c>
+      <c r="B113">
+        <v>1</v>
+      </c>
+      <c r="C113">
+        <v>0</v>
+      </c>
+      <c r="D113">
+        <v>0</v>
+      </c>
+      <c r="F113">
+        <v>16.670000000000002</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>119</v>
+      </c>
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114">
+        <v>1</v>
+      </c>
+      <c r="D114">
+        <v>2</v>
+      </c>
+      <c r="E114">
+        <v>-8.18</v>
+      </c>
+      <c r="F114">
+        <v>2.67</v>
+      </c>
+      <c r="G114">
+        <v>8.51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Manual Analyst Ratings spreadsheet with new data
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6467F8D-C98D-7244-8E79-61A9C6FC21F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA5A1618-27AE-E644-A894-BCC59EBD521C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
   <si>
     <t>Ticker</t>
   </si>
@@ -396,6 +396,12 @@
   </si>
   <si>
     <t>AIFORIA</t>
+  </si>
+  <si>
+    <t>MODU</t>
+  </si>
+  <si>
+    <t>CTH1V</t>
   </si>
 </sst>
 </file>
@@ -767,7 +773,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -3104,6 +3110,37 @@
         <v>8.51</v>
       </c>
     </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A115" t="s">
+        <v>120</v>
+      </c>
+      <c r="B115">
+        <v>0</v>
+      </c>
+      <c r="C115">
+        <v>0</v>
+      </c>
+      <c r="D115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A116" t="s">
+        <v>121</v>
+      </c>
+      <c r="B116">
+        <v>1</v>
+      </c>
+      <c r="C116">
+        <v>0</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+      <c r="F116">
+        <v>6.81</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analyst ratings and add IQMX to tech targets list
</commit_message>
<xml_diff>
--- a/Manual_Analyst_Ratings.xlsx
+++ b/Manual_Analyst_Ratings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/casperkangas/Documents/VS Code/Personal Projects/nordnet-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FAD48BD-14A1-A743-8A1E-47EB9C347E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F752F598-9514-FD4F-82FD-6F419C1E8237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18000" yWindow="800" windowWidth="18000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
+    <workbookView xWindow="18000" yWindow="780" windowWidth="18000" windowHeight="22600" xr2:uid="{E38E31AC-FFDD-624D-BA45-1629BC592AB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
   <si>
     <t>Ticker</t>
   </si>
@@ -402,6 +402,9 @@
   </si>
   <si>
     <t>CTH1V</t>
+  </si>
+  <si>
+    <t>IQMX</t>
   </si>
 </sst>
 </file>
@@ -773,7 +776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1971DA79-8A22-7244-902F-F8980870F481}">
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
@@ -807,19 +810,19 @@
         <v>17</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>-23.52</v>
+        <v>-23.36</v>
       </c>
       <c r="F2">
-        <v>4.1100000000000003</v>
+        <v>4.32</v>
       </c>
       <c r="G2">
-        <v>14.73</v>
+        <v>14.96</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -836,13 +839,13 @@
         <v>2</v>
       </c>
       <c r="E3">
-        <v>-12.88</v>
+        <v>-14.37</v>
       </c>
       <c r="F3">
-        <v>15.49</v>
+        <v>13.51</v>
       </c>
       <c r="G3">
-        <v>69.41</v>
+        <v>66.510000000000005</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -853,19 +856,19 @@
         <v>19</v>
       </c>
       <c r="C4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4">
-        <v>-29.94</v>
+        <v>-32.07</v>
       </c>
       <c r="F4">
-        <v>42.51</v>
+        <v>38.18</v>
       </c>
       <c r="G4">
-        <v>127.62</v>
+        <v>120.7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -873,7 +876,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -881,14 +884,8 @@
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5">
-        <v>-13.39</v>
-      </c>
       <c r="F5">
-        <v>-7.19</v>
-      </c>
-      <c r="G5">
-        <v>-1.57</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -902,16 +899,16 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>-18.579999999999998</v>
+        <v>-19.399999999999999</v>
       </c>
       <c r="F6">
-        <v>-2.8</v>
+        <v>-1.93</v>
       </c>
       <c r="G6">
-        <v>18.739999999999998</v>
+        <v>17.55</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -939,19 +936,19 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
-        <v>-39.020000000000003</v>
+        <v>-45.26</v>
       </c>
       <c r="F8">
-        <v>6.73</v>
+        <v>-7.24</v>
       </c>
       <c r="G8">
-        <v>29.82</v>
+        <v>15.57</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -959,7 +956,7 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -967,14 +964,8 @@
       <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9">
-        <v>-2.12</v>
-      </c>
       <c r="F9">
-        <v>1.96</v>
-      </c>
-      <c r="G9">
-        <v>6.04</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -991,13 +982,13 @@
         <v>5</v>
       </c>
       <c r="E10">
-        <v>-34.86</v>
+        <v>-35.44</v>
       </c>
       <c r="F10">
-        <v>14.12</v>
+        <v>12.95</v>
       </c>
       <c r="G10">
-        <v>47.41</v>
+        <v>46.11</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -1014,13 +1005,13 @@
         <v>1</v>
       </c>
       <c r="E11">
-        <v>-10.79</v>
+        <v>-12.35</v>
       </c>
       <c r="F11">
-        <v>22.26</v>
+        <v>20.12</v>
       </c>
       <c r="G11">
-        <v>64.55</v>
+        <v>61.67</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -1037,13 +1028,13 @@
         <v>3</v>
       </c>
       <c r="E12">
-        <v>-17.03</v>
+        <v>-19.45</v>
       </c>
       <c r="F12">
-        <v>8.91</v>
+        <v>5.97</v>
       </c>
       <c r="G12">
-        <v>32.15</v>
+        <v>28.28</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1060,13 +1051,13 @@
         <v>3</v>
       </c>
       <c r="E13">
-        <v>-37.799999999999997</v>
+        <v>-34.61</v>
       </c>
       <c r="F13">
-        <v>13.25</v>
+        <v>19.05</v>
       </c>
       <c r="G13">
-        <v>92.7</v>
+        <v>102.56</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -1106,13 +1097,13 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>36.28</v>
+        <v>40.229999999999997</v>
       </c>
       <c r="F15">
-        <v>39.380000000000003</v>
+        <v>43.42</v>
       </c>
       <c r="G15">
-        <v>45.68</v>
+        <v>49.9</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -1120,22 +1111,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-0.44</v>
+        <v>-1.21</v>
       </c>
       <c r="F16">
-        <v>10.55</v>
+        <v>9.08</v>
       </c>
       <c r="G16">
-        <v>20.39</v>
+        <v>16.350000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1152,13 +1143,13 @@
         <v>4</v>
       </c>
       <c r="E17">
-        <v>-26.95</v>
+        <v>-26.46</v>
       </c>
       <c r="F17">
-        <v>9.66</v>
+        <v>10.4</v>
       </c>
       <c r="G17">
-        <v>59.53</v>
+        <v>60.61</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1166,22 +1157,22 @@
         <v>23</v>
       </c>
       <c r="B18">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C18">
         <v>7</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18">
-        <v>-21.45</v>
+        <v>-18</v>
       </c>
       <c r="F18">
-        <v>9.77</v>
+        <v>14.6</v>
       </c>
       <c r="G18">
-        <v>32.549999999999997</v>
+        <v>38.380000000000003</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
@@ -1198,13 +1189,13 @@
         <v>2</v>
       </c>
       <c r="E19">
-        <v>-31.93</v>
+        <v>-32.520000000000003</v>
       </c>
       <c r="F19">
-        <v>-4.17</v>
+        <v>-4.99</v>
       </c>
       <c r="G19">
-        <v>6.44</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
@@ -1221,13 +1212,13 @@
         <v>0</v>
       </c>
       <c r="E20">
-        <v>5.65</v>
+        <v>-16.34</v>
       </c>
       <c r="F20">
-        <v>28.23</v>
+        <v>5.67</v>
       </c>
       <c r="G20">
-        <v>45.72</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
@@ -1238,19 +1229,19 @@
         <v>8</v>
       </c>
       <c r="C21">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D21">
         <v>4</v>
       </c>
       <c r="E21">
-        <v>-4.79</v>
+        <v>-4.95</v>
       </c>
       <c r="F21">
-        <v>13.63</v>
+        <v>13.57</v>
       </c>
       <c r="G21">
-        <v>42.53</v>
+        <v>42.29</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1261,19 +1252,19 @@
         <v>5</v>
       </c>
       <c r="C22">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D22">
         <v>7</v>
       </c>
       <c r="E22">
-        <v>-30.12</v>
+        <v>-29.54</v>
       </c>
       <c r="F22">
-        <v>5.57</v>
+        <v>6.95</v>
       </c>
       <c r="G22">
-        <v>36.51</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
@@ -1290,13 +1281,13 @@
         <v>1</v>
       </c>
       <c r="E23">
-        <v>-15.96</v>
+        <v>-15.64</v>
       </c>
       <c r="F23">
-        <v>1.54</v>
+        <v>1.92</v>
       </c>
       <c r="G23">
-        <v>25</v>
+        <v>25.47</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1313,13 +1304,13 @@
         <v>0</v>
       </c>
       <c r="E24">
-        <v>5.49</v>
+        <v>4.82</v>
       </c>
       <c r="F24">
-        <v>10.23</v>
+        <v>9.5399999999999991</v>
       </c>
       <c r="G24">
-        <v>21.31</v>
+        <v>20.55</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -1336,13 +1327,13 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>22.39</v>
+        <v>11.41</v>
       </c>
       <c r="F25">
-        <v>23.88</v>
+        <v>12.77</v>
       </c>
       <c r="G25">
-        <v>25.37</v>
+        <v>14.13</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -1359,7 +1350,7 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>7.53</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -1390,7 +1381,7 @@
         <v>0</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28">
         <v>2.44</v>
@@ -1438,10 +1429,16 @@
         <v>0</v>
       </c>
       <c r="D31">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E31">
+        <v>1.48</v>
       </c>
       <c r="F31">
-        <v>5.49</v>
+        <v>3.59</v>
+      </c>
+      <c r="G31">
+        <v>5.71</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
@@ -1458,13 +1455,13 @@
         <v>0</v>
       </c>
       <c r="E32">
-        <v>8.84</v>
+        <v>6.45</v>
       </c>
       <c r="F32">
-        <v>23.09</v>
+        <v>20.39</v>
       </c>
       <c r="G32">
-        <v>38.520000000000003</v>
+        <v>35.479999999999997</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
@@ -1481,13 +1478,13 @@
         <v>1</v>
       </c>
       <c r="E33">
-        <v>17.98</v>
+        <v>16.54</v>
       </c>
       <c r="F33">
-        <v>20.79</v>
+        <v>19.309999999999999</v>
       </c>
       <c r="G33">
-        <v>23.6</v>
+        <v>22.09</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
@@ -1504,13 +1501,13 @@
         <v>2</v>
       </c>
       <c r="E34">
-        <v>0.93</v>
+        <v>-0.13</v>
       </c>
       <c r="F34">
-        <v>16.600000000000001</v>
+        <v>15.37</v>
       </c>
       <c r="G34">
-        <v>32.799999999999997</v>
+        <v>31.41</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
@@ -1527,13 +1524,13 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>1.94</v>
+        <v>0</v>
       </c>
       <c r="F35">
-        <v>20</v>
+        <v>17.71</v>
       </c>
       <c r="G35">
-        <v>35.92</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
@@ -1544,19 +1541,19 @@
         <v>1</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36">
         <v>0</v>
       </c>
       <c r="E36">
-        <v>22.75</v>
+        <v>15.04</v>
       </c>
       <c r="F36">
-        <v>41.96</v>
+        <v>23.89</v>
       </c>
       <c r="G36">
-        <v>63.67</v>
+        <v>32.74</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -1573,13 +1570,13 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>7.66</v>
+        <v>6.59</v>
       </c>
       <c r="F37">
-        <v>9.8800000000000008</v>
+        <v>8.7899999999999991</v>
       </c>
       <c r="G37">
-        <v>10.99</v>
+        <v>9.89</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -1596,13 +1593,13 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>3.32</v>
+        <v>1.45</v>
       </c>
       <c r="F38">
-        <v>24.39</v>
+        <v>22.14</v>
       </c>
       <c r="G38">
-        <v>40.22</v>
+        <v>37.68</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
@@ -1619,13 +1616,13 @@
         <v>0</v>
       </c>
       <c r="E39">
-        <v>7.0000000000000007E-2</v>
+        <v>-0.74</v>
       </c>
       <c r="F39">
-        <v>17.010000000000002</v>
+        <v>16.07</v>
       </c>
       <c r="G39">
-        <v>40.85</v>
+        <v>39.71</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
@@ -1642,13 +1639,13 @@
         <v>3</v>
       </c>
       <c r="E40">
-        <v>-7.14</v>
+        <v>-8.73</v>
       </c>
       <c r="F40">
-        <v>7.14</v>
+        <v>5.31</v>
       </c>
       <c r="G40">
-        <v>27.68</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -1668,10 +1665,10 @@
         <v>-26.55</v>
       </c>
       <c r="F41">
-        <v>7.34</v>
+        <v>7.72</v>
       </c>
       <c r="G41">
-        <v>43.13</v>
+        <v>41.24</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -1688,13 +1685,13 @@
         <v>0</v>
       </c>
       <c r="E42">
-        <v>-0.57999999999999996</v>
+        <v>-1.9</v>
       </c>
       <c r="F42">
-        <v>14.11</v>
+        <v>12.88</v>
       </c>
       <c r="G42">
-        <v>31.49</v>
+        <v>29.75</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
@@ -1711,13 +1708,13 @@
         <v>1</v>
       </c>
       <c r="E43">
-        <v>-36.880000000000003</v>
+        <v>-37.369999999999997</v>
       </c>
       <c r="F43">
-        <v>4.16</v>
+        <v>4.68</v>
       </c>
       <c r="G43">
-        <v>33.17</v>
+        <v>32.24</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -1734,7 +1731,7 @@
         <v>1</v>
       </c>
       <c r="F44">
-        <v>13.16</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -1751,7 +1748,7 @@
         <v>1</v>
       </c>
       <c r="F45">
-        <v>44.85</v>
+        <v>37.93</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
@@ -1768,13 +1765,13 @@
         <v>0</v>
       </c>
       <c r="E46">
-        <v>4.21</v>
+        <v>-1.05</v>
       </c>
       <c r="F46">
-        <v>7.54</v>
+        <v>2.11</v>
       </c>
       <c r="G46">
-        <v>10.86</v>
+        <v>5.26</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
@@ -1791,7 +1788,7 @@
         <v>1</v>
       </c>
       <c r="F47">
-        <v>-6.98</v>
+        <v>-15.09</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
@@ -1799,22 +1796,22 @@
         <v>53</v>
       </c>
       <c r="B48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C48">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D48">
         <v>2</v>
       </c>
       <c r="E48">
-        <v>-16.829999999999998</v>
+        <v>-22.16</v>
       </c>
       <c r="F48">
-        <v>-1.2</v>
+        <v>-5.09</v>
       </c>
       <c r="G48">
-        <v>6.45</v>
+        <v>19.760000000000002</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
@@ -1822,22 +1819,13 @@
         <v>54</v>
       </c>
       <c r="B49">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C49">
         <v>0</v>
       </c>
       <c r="D49">
         <v>0</v>
-      </c>
-      <c r="E49">
-        <v>-7.08</v>
-      </c>
-      <c r="F49">
-        <v>-4.87</v>
-      </c>
-      <c r="G49">
-        <v>-2.65</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -1854,7 +1842,7 @@
         <v>1</v>
       </c>
       <c r="F50">
-        <v>11.61</v>
+        <v>10.039999999999999</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
@@ -1862,16 +1850,13 @@
         <v>56</v>
       </c>
       <c r="B51">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C51">
         <v>0</v>
       </c>
       <c r="D51">
         <v>0</v>
-      </c>
-      <c r="F51">
-        <v>20.37</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
@@ -1888,7 +1873,7 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>476.92</v>
+        <v>482.52</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
@@ -1905,7 +1890,7 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>63.93</v>
+        <v>64.709999999999994</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
@@ -1922,7 +1907,7 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>27.93</v>
+        <v>23.13</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
@@ -1936,10 +1921,7 @@
         <v>0</v>
       </c>
       <c r="D55">
-        <v>1</v>
-      </c>
-      <c r="F55">
-        <v>0.28999999999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.2">
@@ -1956,13 +1938,13 @@
         <v>2</v>
       </c>
       <c r="E56">
-        <v>-6.73</v>
+        <v>4.4800000000000004</v>
       </c>
       <c r="F56">
-        <v>-3</v>
+        <v>7.46</v>
       </c>
       <c r="G56">
-        <v>2.6</v>
+        <v>13.43</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
@@ -1979,13 +1961,13 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>-2.6</v>
+        <v>-3.73</v>
       </c>
       <c r="F57">
-        <v>1.89</v>
+        <v>0.7</v>
       </c>
       <c r="G57">
-        <v>6.26</v>
+        <v>5.0199999999999996</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
@@ -1996,13 +1978,13 @@
         <v>0</v>
       </c>
       <c r="C58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D58">
         <v>0</v>
       </c>
       <c r="F58">
-        <v>-0.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -2010,22 +1992,22 @@
         <v>64</v>
       </c>
       <c r="B59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C59">
         <v>0</v>
       </c>
       <c r="D59">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E59">
-        <v>3.41</v>
+        <v>7.53</v>
       </c>
       <c r="F59">
-        <v>14.36</v>
+        <v>10.51</v>
       </c>
       <c r="G59">
-        <v>24.7</v>
+        <v>16.489999999999998</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
@@ -2042,13 +2024,13 @@
         <v>1</v>
       </c>
       <c r="E60">
-        <v>-8.02</v>
+        <v>-7.8</v>
       </c>
       <c r="F60">
-        <v>3.44</v>
+        <v>3.69</v>
       </c>
       <c r="G60">
-        <v>13.21</v>
+        <v>13.48</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
@@ -2056,7 +2038,7 @@
         <v>66</v>
       </c>
       <c r="B61">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -2065,13 +2047,13 @@
         <v>0</v>
       </c>
       <c r="E61">
-        <v>10.82</v>
+        <v>12.78</v>
       </c>
       <c r="F61">
-        <v>14.34</v>
+        <v>14.41</v>
       </c>
       <c r="G61">
-        <v>19.95</v>
+        <v>17.79</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
@@ -2088,13 +2070,13 @@
         <v>3</v>
       </c>
       <c r="E62">
-        <v>-20.34</v>
+        <v>-17.829999999999998</v>
       </c>
       <c r="F62">
-        <v>-8.09</v>
+        <v>-5.18</v>
       </c>
       <c r="G62">
-        <v>-1.96</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
@@ -2111,13 +2093,13 @@
         <v>0</v>
       </c>
       <c r="E63">
-        <v>4.88</v>
+        <v>-2.71</v>
       </c>
       <c r="F63">
-        <v>13.34</v>
+        <v>9.57</v>
       </c>
       <c r="G63">
-        <v>21.95</v>
+        <v>17.649999999999999</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
@@ -2139,16 +2121,13 @@
         <v>70</v>
       </c>
       <c r="B65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C65">
         <v>0</v>
       </c>
       <c r="D65">
         <v>0</v>
-      </c>
-      <c r="F65">
-        <v>15.65</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
@@ -2165,13 +2144,13 @@
         <v>0</v>
       </c>
       <c r="E66">
-        <v>0.86</v>
+        <v>-2.08</v>
       </c>
       <c r="F66">
-        <v>21.24</v>
+        <v>17.71</v>
       </c>
       <c r="G66">
-        <v>41.63</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
@@ -2188,13 +2167,13 @@
         <v>0</v>
       </c>
       <c r="E67">
-        <v>-7.22</v>
+        <v>-10.74</v>
       </c>
       <c r="F67">
-        <v>2.41</v>
+        <v>-1.49</v>
       </c>
       <c r="G67">
-        <v>9.9700000000000006</v>
+        <v>5.79</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
@@ -2216,7 +2195,7 @@
         <v>72</v>
       </c>
       <c r="B69">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -2224,8 +2203,14 @@
       <c r="D69">
         <v>0</v>
       </c>
+      <c r="E69">
+        <v>18.059999999999999</v>
+      </c>
       <c r="F69">
-        <v>36.51</v>
+        <v>31.08</v>
+      </c>
+      <c r="G69">
+        <v>44.1</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
@@ -2233,7 +2218,7 @@
         <v>73</v>
       </c>
       <c r="B70">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C70">
         <v>0</v>
@@ -2241,14 +2226,8 @@
       <c r="D70">
         <v>0</v>
       </c>
-      <c r="E70">
-        <v>16.850000000000001</v>
-      </c>
       <c r="F70">
-        <v>19.93</v>
-      </c>
-      <c r="G70">
-        <v>23</v>
+        <v>24.22</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
@@ -2265,7 +2244,7 @@
         <v>0</v>
       </c>
       <c r="F71">
-        <v>23.97</v>
+        <v>14.94</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
@@ -2282,13 +2261,13 @@
         <v>0</v>
       </c>
       <c r="E72">
-        <v>0.6</v>
+        <v>-3.91</v>
       </c>
       <c r="F72">
-        <v>16.79</v>
+        <v>11.56</v>
       </c>
       <c r="G72">
-        <v>27.88</v>
+        <v>22.15</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
@@ -2305,13 +2284,13 @@
         <v>5</v>
       </c>
       <c r="E73">
-        <v>-49.87</v>
+        <v>-49.04</v>
       </c>
       <c r="F73">
-        <v>-15.49</v>
+        <v>-14.1</v>
       </c>
       <c r="G73">
-        <v>17.190000000000001</v>
+        <v>19.13</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
@@ -2328,13 +2307,13 @@
         <v>3</v>
       </c>
       <c r="E74">
-        <v>-13.14</v>
+        <v>-14.05</v>
       </c>
       <c r="F74">
-        <v>-6.34</v>
+        <v>-7.32</v>
       </c>
       <c r="G74">
-        <v>5.74</v>
+        <v>4.63</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
@@ -2351,13 +2330,13 @@
         <v>0</v>
       </c>
       <c r="E75">
-        <v>8.49</v>
+        <v>8.9</v>
       </c>
       <c r="F75">
-        <v>17.920000000000002</v>
+        <v>18.37</v>
       </c>
       <c r="G75">
-        <v>27.36</v>
+        <v>27.84</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
@@ -2388,7 +2367,7 @@
         <v>1</v>
       </c>
       <c r="F77">
-        <v>13.15</v>
+        <v>12.04</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.2">
@@ -2405,13 +2384,13 @@
         <v>1</v>
       </c>
       <c r="E78">
-        <v>-2.72</v>
+        <v>-6.72</v>
       </c>
       <c r="F78">
-        <v>3.5</v>
+        <v>-0.75</v>
       </c>
       <c r="G78">
-        <v>8.9499999999999993</v>
+        <v>4.4800000000000004</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
@@ -2428,13 +2407,13 @@
         <v>0</v>
       </c>
       <c r="E79">
-        <v>13.28</v>
+        <v>11.75</v>
       </c>
       <c r="F79">
-        <v>22.66</v>
+        <v>21</v>
       </c>
       <c r="G79">
-        <v>44.53</v>
+        <v>42.58</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
@@ -2442,7 +2421,7 @@
         <v>85</v>
       </c>
       <c r="B80">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -2451,13 +2430,13 @@
         <v>2</v>
       </c>
       <c r="E80">
-        <v>-9.59</v>
+        <v>-2.44</v>
       </c>
       <c r="F80">
-        <v>1.92</v>
+        <v>1.08</v>
       </c>
       <c r="G80">
-        <v>17.809999999999999</v>
+        <v>5.69</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
@@ -2474,13 +2453,13 @@
         <v>0</v>
       </c>
       <c r="E81">
-        <v>4.03</v>
+        <v>2.04</v>
       </c>
       <c r="F81">
-        <v>15.28</v>
+        <v>13.07</v>
       </c>
       <c r="G81">
-        <v>23.54</v>
+        <v>21.17</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
@@ -2496,9 +2475,6 @@
       <c r="D82">
         <v>2</v>
       </c>
-      <c r="F82">
-        <v>1.63</v>
-      </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
@@ -2514,7 +2490,7 @@
         <v>0</v>
       </c>
       <c r="F83">
-        <v>22.03</v>
+        <v>24.14</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
@@ -2531,13 +2507,13 @@
         <v>0</v>
       </c>
       <c r="E84">
-        <v>10.24</v>
+        <v>8.43</v>
       </c>
       <c r="F84">
-        <v>31.85</v>
+        <v>29.68</v>
       </c>
       <c r="G84">
-        <v>55.9</v>
+        <v>53.34</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
@@ -2554,13 +2530,13 @@
         <v>5</v>
       </c>
       <c r="E85">
-        <v>-27.1</v>
+        <v>-27.39</v>
       </c>
       <c r="F85">
-        <v>-20.010000000000002</v>
+        <v>-20.329999999999998</v>
       </c>
       <c r="G85">
-        <v>-4.82</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.2">
@@ -2577,7 +2553,7 @@
         <v>2</v>
       </c>
       <c r="F86">
-        <v>-4.26</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
@@ -2591,7 +2567,10 @@
         <v>0</v>
       </c>
       <c r="D87">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="F87">
+        <v>-19.54</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
@@ -2608,7 +2587,7 @@
         <v>1</v>
       </c>
       <c r="F88">
-        <v>1.4</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.2">
@@ -2625,13 +2604,13 @@
         <v>0</v>
       </c>
       <c r="E89">
-        <v>9.3800000000000008</v>
+        <v>9.5500000000000007</v>
       </c>
       <c r="F89">
-        <v>19.22</v>
+        <v>19.41</v>
       </c>
       <c r="G89">
-        <v>43.23</v>
+        <v>43.45</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
@@ -2639,7 +2618,7 @@
         <v>95</v>
       </c>
       <c r="B90">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C90">
         <v>1</v>
@@ -2648,13 +2627,13 @@
         <v>0</v>
       </c>
       <c r="E90">
-        <v>1.48</v>
+        <v>7.41</v>
       </c>
       <c r="F90">
-        <v>7.93</v>
+        <v>11.11</v>
       </c>
       <c r="G90">
-        <v>11.11</v>
+        <v>14.81</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.2">
@@ -2671,7 +2650,7 @@
         <v>1</v>
       </c>
       <c r="F91">
-        <v>-16.670000000000002</v>
+        <v>-13.79</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.2">
@@ -2702,16 +2681,16 @@
         <v>98</v>
       </c>
       <c r="B93">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C93">
         <v>0</v>
       </c>
       <c r="D93">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F93">
-        <v>-3.7</v>
+        <v>13.64</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
@@ -2728,7 +2707,7 @@
         <v>0</v>
       </c>
       <c r="F94">
-        <v>25</v>
+        <v>20.16</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
@@ -2744,14 +2723,8 @@
       <c r="D95">
         <v>3</v>
       </c>
-      <c r="E95">
-        <v>0.28999999999999998</v>
-      </c>
       <c r="F95">
-        <v>6.06</v>
-      </c>
-      <c r="G95">
-        <v>14.61</v>
+        <v>9.7200000000000006</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
@@ -2768,7 +2741,7 @@
         <v>0</v>
       </c>
       <c r="F96">
-        <v>-4.28</v>
+        <v>5.69</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
@@ -2785,7 +2758,7 @@
         <v>1</v>
       </c>
       <c r="F97">
-        <v>-1.64</v>
+        <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
@@ -2802,13 +2775,13 @@
         <v>1</v>
       </c>
       <c r="E98">
-        <v>-2.2999999999999998</v>
+        <v>-5.53</v>
       </c>
       <c r="F98">
-        <v>1.72</v>
+        <v>-0.57999999999999996</v>
       </c>
       <c r="G98">
-        <v>5.75</v>
+        <v>5.99</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.2">
@@ -2825,13 +2798,13 @@
         <v>0</v>
       </c>
       <c r="E99">
-        <v>105.76</v>
+        <v>110.53</v>
       </c>
       <c r="F99">
-        <v>943.21</v>
+        <v>967.37</v>
       </c>
       <c r="G99">
-        <v>2309.4699999999998</v>
+        <v>2365.2600000000002</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.2">
@@ -2848,7 +2821,7 @@
         <v>0</v>
       </c>
       <c r="F100">
-        <v>16.399999999999999</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.2">
@@ -2865,7 +2838,7 @@
         <v>0</v>
       </c>
       <c r="F101">
-        <v>42.86</v>
+        <v>30.43</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.2">
@@ -2882,7 +2855,7 @@
         <v>0</v>
       </c>
       <c r="F102">
-        <v>28.68</v>
+        <v>23.13</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.2">
@@ -2899,13 +2872,13 @@
         <v>0</v>
       </c>
       <c r="E103">
-        <v>128.05000000000001</v>
+        <v>102.2</v>
       </c>
       <c r="F103">
-        <v>147.43</v>
+        <v>119.19</v>
       </c>
       <c r="G103">
-        <v>156.56</v>
+        <v>127.27</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.2">
@@ -2913,22 +2886,22 @@
         <v>109</v>
       </c>
       <c r="B104">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C104">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D104">
         <v>0</v>
       </c>
       <c r="E104">
-        <v>7.59</v>
+        <v>13.25</v>
       </c>
       <c r="F104">
-        <v>28.61</v>
+        <v>25.45</v>
       </c>
       <c r="G104">
-        <v>51.9</v>
+        <v>49.35</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.2">
@@ -2945,7 +2918,7 @@
         <v>1</v>
       </c>
       <c r="F105">
-        <v>15.38</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.2">
@@ -2962,13 +2935,13 @@
         <v>0</v>
       </c>
       <c r="E106">
-        <v>40.9</v>
+        <v>31.63</v>
       </c>
       <c r="F106">
-        <v>63.37</v>
+        <v>52.61</v>
       </c>
       <c r="G106">
-        <v>114.09</v>
+        <v>100</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.2">
@@ -2985,7 +2958,7 @@
         <v>1</v>
       </c>
       <c r="F107">
-        <v>-12.5</v>
+        <v>-17.86</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.2">
@@ -3002,13 +2975,13 @@
         <v>2</v>
       </c>
       <c r="E108">
-        <v>10.98</v>
+        <v>6.74</v>
       </c>
       <c r="F108">
-        <v>28.5</v>
+        <v>23.6</v>
       </c>
       <c r="G108">
-        <v>63.55</v>
+        <v>57.3</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.2">
@@ -3025,13 +2998,13 @@
         <v>0</v>
       </c>
       <c r="E109">
-        <v>19.05</v>
+        <v>4.9400000000000004</v>
       </c>
       <c r="F109">
-        <v>24.06</v>
+        <v>15.56</v>
       </c>
       <c r="G109">
-        <v>30.33</v>
+        <v>23.46</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.2">
@@ -3048,13 +3021,13 @@
         <v>0</v>
       </c>
       <c r="E110">
-        <v>23.32</v>
+        <v>16.5</v>
       </c>
       <c r="F110">
-        <v>30.72</v>
+        <v>35.92</v>
       </c>
       <c r="G110">
-        <v>34.53</v>
+        <v>45.63</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.2">
@@ -3099,7 +3072,7 @@
         <v>0</v>
       </c>
       <c r="F113">
-        <v>14.29</v>
+        <v>12.45</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.2">
@@ -3116,13 +3089,13 @@
         <v>2</v>
       </c>
       <c r="E114">
-        <v>-7.72</v>
+        <v>-0.36</v>
       </c>
       <c r="F114">
-        <v>3.19</v>
+        <v>11.41</v>
       </c>
       <c r="G114">
-        <v>9.06</v>
+        <v>17.75</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.2">
@@ -3153,7 +3126,21 @@
         <v>0</v>
       </c>
       <c r="F116">
-        <v>-0.86</v>
+        <v>-8.73</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A117" t="s">
+        <v>122</v>
+      </c>
+      <c r="B117">
+        <v>0</v>
+      </c>
+      <c r="C117">
+        <v>0</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>